<commit_message>
Sales, commercials and support documents for AML/CFT, IC registers, BIR and EOPT, integrations, dealer programmes, branding, My Work and the Report Builder; new optional price lines to confirm by management; builds of the brochures, deck and workbooks
</commit_message>
<xml_diff>
--- a/docs/package/02_Commercials/BrokerVerse_Commercials_and_Pricing.xlsx
+++ b/docs/package/02_Commercials/BrokerVerse_Commercials_and_Pricing.xlsx
@@ -56,14 +56,20 @@
     <definedName name="Int_Std_Days">Inputs!$B$59</definedName>
     <definedName name="Int_Cx_Days">Inputs!$B$60</definedName>
     <definedName name="Report_Days">Inputs!$B$61</definedName>
-    <definedName name="NP_Small_USD">Inputs!$B$75</definedName>
-    <definedName name="NP_Med_USD">Inputs!$B$76</definedName>
-    <definedName name="PreProd_Factor">Inputs!$B$77</definedName>
-    <definedName name="PreProd_GoLive_Months">Inputs!$B$78</definedName>
-    <definedName name="PreProd_Rel_Months">Inputs!$B$79</definedName>
-    <definedName name="Major_Rel_Year">Inputs!$B$80</definedName>
-    <definedName name="Azure_Factor">Inputs!$B$88</definedName>
-    <definedName name="Local_Factor">Inputs!$B$89</definedName>
+    <definedName name="Conn_Golive_Days">Inputs!$B$62</definedName>
+    <definedName name="AML_Act_Days">Inputs!$B$63</definedName>
+    <definedName name="IC_Act_Days">Inputs!$B$64</definedName>
+    <definedName name="BIR_Act_Days">Inputs!$B$65</definedName>
+    <definedName name="Dealer_Prog_Days">Inputs!$B$66</definedName>
+    <definedName name="Brand_Pack_Days">Inputs!$B$67</definedName>
+    <definedName name="NP_Small_USD">Inputs!$B$81</definedName>
+    <definedName name="NP_Med_USD">Inputs!$B$82</definedName>
+    <definedName name="PreProd_Factor">Inputs!$B$83</definedName>
+    <definedName name="PreProd_GoLive_Months">Inputs!$B$84</definedName>
+    <definedName name="PreProd_Rel_Months">Inputs!$B$85</definedName>
+    <definedName name="Major_Rel_Year">Inputs!$B$86</definedName>
+    <definedName name="Azure_Factor">Inputs!$B$94</definedName>
+    <definedName name="Local_Factor">Inputs!$B$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3216,7 +3222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N100"/>
+  <dimension ref="A1:N106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4784,7 +4790,7 @@
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>Estimate: e.g. one insurer API, SMS gateway, payment gateway variant.</t>
+          <t>Estimate: a new kind of interface not covered by the delivered connectors, e.g. a payment gateway variant or an accounting package feed.</t>
         </is>
       </c>
       <c r="E59" s="8" t="n"/>
@@ -4858,57 +4864,87 @@
       <c r="M61" s="8" t="n"/>
       <c r="N61" s="9" t="n"/>
     </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>Go-live of a delivered connector with one partner (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: SMS gateway, CTPL provider, one insurer API mapping, one bank file layout or the BIR EIS: configuration, credentials check, live test, support of the partner acceptance. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="n"/>
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="8" t="n"/>
+      <c r="H62" s="8" t="n"/>
+      <c r="I62" s="8" t="n"/>
+      <c r="J62" s="8" t="n"/>
+      <c r="K62" s="8" t="n"/>
+      <c r="L62" s="8" t="n"/>
+      <c r="M62" s="8" t="n"/>
+      <c r="N62" s="9" t="n"/>
+    </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>Infrastructure: AWS reference cost per month of the Production environment (USD)</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="n"/>
-      <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
-      <c r="E63" s="7" t="n"/>
-      <c r="F63" s="7" t="n"/>
-      <c r="G63" s="7" t="n"/>
-      <c r="H63" s="7" t="n"/>
-      <c r="I63" s="7" t="n"/>
-      <c r="J63" s="7" t="n"/>
-      <c r="K63" s="7" t="n"/>
-      <c r="L63" s="7" t="n"/>
-      <c r="M63" s="7" t="n"/>
-      <c r="N63" s="7" t="n"/>
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>Activation of the AML/CFT toolkit (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: risk factors and rules workshop with the compliance officer, settings, first list loads, provider set-up, AMLC test file. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="8" t="n"/>
+      <c r="H63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="J63" s="8" t="n"/>
+      <c r="K63" s="8" t="n"/>
+      <c r="L63" s="8" t="n"/>
+      <c r="M63" s="8" t="n"/>
+      <c r="N63" s="9" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>Activation of the IC compliance registers (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: licence and fit and proper register load, insurer certificates, complaints and breach settings, IC statement account mapping to the broker chart. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="8" t="n"/>
       <c r="G64" s="8" t="n"/>
       <c r="H64" s="8" t="n"/>
       <c r="I64" s="8" t="n"/>
@@ -4921,26 +4957,24 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Application containers (API, web, scheduler)</t>
-        </is>
-      </c>
-      <c r="B65" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="C65" s="16" t="n">
-        <v>135</v>
-      </c>
-      <c r="D65" s="16" t="n">
-        <v>180</v>
-      </c>
-      <c r="E65" s="16" t="n">
-        <v>360</v>
-      </c>
-      <c r="F65" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 2/3/4/8 containers of 1 vCPU, 2 GB (Fargate, Singapore).</t>
-        </is>
-      </c>
+          <t>Activation of the BIR pack (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: BIR and EOPT invoice settings with the tax adviser, ATC mapping, DAT file dry run, CAS books pack. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="8" t="n"/>
       <c r="G65" s="8" t="n"/>
       <c r="H65" s="8" t="n"/>
       <c r="I65" s="8" t="n"/>
@@ -4953,26 +4987,24 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Managed PostgreSQL 16 (instance and storage)</t>
-        </is>
-      </c>
-      <c r="B66" s="16" t="n">
-        <v>85</v>
-      </c>
-      <c r="C66" s="16" t="n">
-        <v>320</v>
-      </c>
-      <c r="D66" s="16" t="n">
-        <v>640</v>
-      </c>
-      <c r="E66" s="16" t="n">
-        <v>1280</v>
-      </c>
-      <c r="F66" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: db.t4g.medium single-AZ / db.m7g.large Multi-AZ / m7g.xlarge Multi-AZ / m7g.2xlarge Multi-AZ (S20). Large and Enterprise: high availability.</t>
-        </is>
-      </c>
+          <t>Set-up of one dealer programme (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: channels, rates, subsidy, bank letter and the first upload. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="n"/>
+      <c r="F66" s="8" t="n"/>
       <c r="G66" s="8" t="n"/>
       <c r="H66" s="8" t="n"/>
       <c r="I66" s="8" t="n"/>
@@ -4985,26 +5017,24 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Object storage and backups (documents, snapshots)</t>
-        </is>
-      </c>
-      <c r="B67" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="C67" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="D67" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="E67" s="16" t="n">
-        <v>180</v>
-      </c>
-      <c r="F67" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: S3 and snapshot storage, growing with policies and uploads.</t>
-        </is>
-      </c>
+          <t>Client brand pack (to confirm by management)</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: theme, sign-in picture, document and e-mail branding, e-signature mapping, exported pack. To confirm by management.</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="n"/>
+      <c r="F67" s="8" t="n"/>
       <c r="G67" s="8" t="n"/>
       <c r="H67" s="8" t="n"/>
       <c r="I67" s="8" t="n"/>
@@ -5014,91 +5044,55 @@
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="9" t="n"/>
     </row>
-    <row r="68">
-      <c r="A68" s="10" t="inlineStr">
-        <is>
-          <t>Network (load balancer, CDN, data transfer)</t>
-        </is>
-      </c>
-      <c r="B68" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="C68" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="D68" s="16" t="n">
-        <v>120</v>
-      </c>
-      <c r="E68" s="16" t="n">
-        <v>220</v>
-      </c>
-      <c r="F68" s="15" t="inlineStr">
-        <is>
-          <t>Estimate.</t>
-        </is>
-      </c>
-      <c r="G68" s="8" t="n"/>
-      <c r="H68" s="8" t="n"/>
-      <c r="I68" s="8" t="n"/>
-      <c r="J68" s="8" t="n"/>
-      <c r="K68" s="8" t="n"/>
-      <c r="L68" s="8" t="n"/>
-      <c r="M68" s="8" t="n"/>
-      <c r="N68" s="9" t="n"/>
-    </row>
     <row r="69">
-      <c r="A69" s="10" t="inlineStr">
-        <is>
-          <t>Security and monitoring (WAF, logs, alarms, secrets, keys)</t>
-        </is>
-      </c>
-      <c r="B69" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="C69" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="D69" s="16" t="n">
-        <v>110</v>
-      </c>
-      <c r="E69" s="16" t="n">
-        <v>200</v>
-      </c>
-      <c r="F69" s="15" t="inlineStr">
-        <is>
-          <t>Estimate.</t>
-        </is>
-      </c>
-      <c r="G69" s="8" t="n"/>
-      <c r="H69" s="8" t="n"/>
-      <c r="I69" s="8" t="n"/>
-      <c r="J69" s="8" t="n"/>
-      <c r="K69" s="8" t="n"/>
-      <c r="L69" s="8" t="n"/>
-      <c r="M69" s="8" t="n"/>
-      <c r="N69" s="9" t="n"/>
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>Infrastructure: AWS reference cost per month of the Production environment (USD)</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="n"/>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n"/>
+      <c r="G69" s="7" t="n"/>
+      <c r="H69" s="7" t="n"/>
+      <c r="I69" s="7" t="n"/>
+      <c r="J69" s="7" t="n"/>
+      <c r="K69" s="7" t="n"/>
+      <c r="L69" s="7" t="n"/>
+      <c r="M69" s="7" t="n"/>
+      <c r="N69" s="7" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="inlineStr">
-        <is>
-          <t>Disaster recovery copy (cross-region backups)</t>
-        </is>
-      </c>
-      <c r="B70" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C70" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="16" t="n">
-        <v>400</v>
-      </c>
-      <c r="F70" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: Enterprise only; optional for others. Not part of Pre-Prod.</t>
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Basis</t>
         </is>
       </c>
       <c r="G70" s="8" t="n"/>
@@ -5111,71 +5105,124 @@
       <c r="N70" s="9" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="18" t="inlineStr">
-        <is>
-          <t>Production reference cost per month (USD)</t>
-        </is>
-      </c>
-      <c r="B71" s="21">
-        <f>SUM(B65:B70)</f>
-        <v/>
-      </c>
-      <c r="C71" s="21">
-        <f>SUM(C65:C70)</f>
-        <v/>
-      </c>
-      <c r="D71" s="21">
-        <f>SUM(D65:D70)</f>
-        <v/>
-      </c>
-      <c r="E71" s="21">
-        <f>SUM(E65:E70)</f>
-        <v/>
-      </c>
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Application containers (API, web, scheduler)</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="C71" s="16" t="n">
+        <v>135</v>
+      </c>
+      <c r="D71" s="16" t="n">
+        <v>180</v>
+      </c>
+      <c r="E71" s="16" t="n">
+        <v>360</v>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 2/3/4/8 containers of 1 vCPU, 2 GB (Fargate, Singapore).</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="n"/>
+      <c r="H71" s="8" t="n"/>
+      <c r="I71" s="8" t="n"/>
+      <c r="J71" s="8" t="n"/>
+      <c r="K71" s="8" t="n"/>
+      <c r="L71" s="8" t="n"/>
+      <c r="M71" s="8" t="n"/>
+      <c r="N71" s="9" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>Managed PostgreSQL 16 (instance and storage)</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="n">
+        <v>85</v>
+      </c>
+      <c r="C72" s="16" t="n">
+        <v>320</v>
+      </c>
+      <c r="D72" s="16" t="n">
+        <v>640</v>
+      </c>
+      <c r="E72" s="16" t="n">
+        <v>1280</v>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: db.t4g.medium single-AZ / db.m7g.large Multi-AZ / m7g.xlarge Multi-AZ / m7g.2xlarge Multi-AZ (S20). Large and Enterprise: high availability.</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="n"/>
+      <c r="H72" s="8" t="n"/>
+      <c r="I72" s="8" t="n"/>
+      <c r="J72" s="8" t="n"/>
+      <c r="K72" s="8" t="n"/>
+      <c r="L72" s="8" t="n"/>
+      <c r="M72" s="8" t="n"/>
+      <c r="N72" s="9" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>Infrastructure: non-production environment sizes and Pre-Prod use</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="n"/>
-      <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
-      <c r="E73" s="7" t="n"/>
-      <c r="F73" s="7" t="n"/>
-      <c r="G73" s="7" t="n"/>
-      <c r="H73" s="7" t="n"/>
-      <c r="I73" s="7" t="n"/>
-      <c r="J73" s="7" t="n"/>
-      <c r="K73" s="7" t="n"/>
-      <c r="L73" s="7" t="n"/>
-      <c r="M73" s="7" t="n"/>
-      <c r="N73" s="7" t="n"/>
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Object storage and backups (documents, snapshots)</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C73" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D73" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="E73" s="16" t="n">
+        <v>180</v>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: S3 and snapshot storage, growing with policies and uploads.</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+      <c r="J73" s="8" t="n"/>
+      <c r="K73" s="8" t="n"/>
+      <c r="L73" s="8" t="n"/>
+      <c r="M73" s="8" t="n"/>
+      <c r="N73" s="9" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="n"/>
-      <c r="F74" s="8" t="n"/>
+      <c r="A74" s="10" t="inlineStr">
+        <is>
+          <t>Network (load balancer, CDN, data transfer)</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="C74" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="D74" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="E74" s="16" t="n">
+        <v>220</v>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>Estimate.</t>
+        </is>
+      </c>
       <c r="G74" s="8" t="n"/>
       <c r="H74" s="8" t="n"/>
       <c r="I74" s="8" t="n"/>
@@ -5188,24 +5235,26 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>Non-production environment, small: cloud cost per month</t>
+          <t>Security and monitoring (WAF, logs, alarms, secrets, keys)</t>
         </is>
       </c>
       <c r="B75" s="16" t="n">
-        <v>150</v>
-      </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 1 container of 1 vCPU, 2 GB; PostgreSQL db.t4g.medium single-AZ, 50 GB; file store; backups 7 to 14 days. Dev in every tier; UAT of Small and Medium brokers.</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="n"/>
-      <c r="F75" s="8" t="n"/>
+        <v>35</v>
+      </c>
+      <c r="C75" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="D75" s="16" t="n">
+        <v>110</v>
+      </c>
+      <c r="E75" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>Estimate.</t>
+        </is>
+      </c>
       <c r="G75" s="8" t="n"/>
       <c r="H75" s="8" t="n"/>
       <c r="I75" s="8" t="n"/>
@@ -5218,24 +5267,26 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Non-production environment, medium: cloud cost per month</t>
+          <t>Disaster recovery copy (cross-region backups)</t>
         </is>
       </c>
       <c r="B76" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 2 containers of 1 vCPU, 2 GB (the second for the UAT performance test); db.t4g.large single-AZ, 100 GB; file store; load balancer. SIT and UAT of Large and Enterprise brokers.</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="n"/>
-      <c r="F76" s="8" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="C76" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: Enterprise only; optional for others. Not part of Pre-Prod.</t>
+        </is>
+      </c>
       <c r="G76" s="8" t="n"/>
       <c r="H76" s="8" t="n"/>
       <c r="I76" s="8" t="n"/>
@@ -5246,112 +5297,67 @@
       <c r="N76" s="9" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="inlineStr">
-        <is>
-          <t>Pre-Prod cloud cost relative to Production (without the DR copy)</t>
-        </is>
-      </c>
-      <c r="B77" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: Pre-Prod is restored from a production backup and runs at production topology and size, so the rehearsal measures real timings.</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="n"/>
-      <c r="F77" s="8" t="n"/>
-      <c r="G77" s="8" t="n"/>
-      <c r="H77" s="8" t="n"/>
-      <c r="I77" s="8" t="n"/>
-      <c r="J77" s="8" t="n"/>
-      <c r="K77" s="8" t="n"/>
-      <c r="L77" s="8" t="n"/>
-      <c r="M77" s="8" t="n"/>
-      <c r="N77" s="9" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="10" t="inlineStr">
-        <is>
-          <t>Pre-Prod months of use around go-live</t>
-        </is>
-      </c>
-      <c r="B78" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: created before the cutover rehearsal and removed after hypercare (1 to 2 months). Billed per month of use.</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="n"/>
-      <c r="F78" s="8" t="n"/>
-      <c r="G78" s="8" t="n"/>
-      <c r="H78" s="8" t="n"/>
-      <c r="I78" s="8" t="n"/>
-      <c r="J78" s="8" t="n"/>
-      <c r="K78" s="8" t="n"/>
-      <c r="L78" s="8" t="n"/>
-      <c r="M78" s="8" t="n"/>
-      <c r="N78" s="9" t="n"/>
+      <c r="A77" s="18" t="inlineStr">
+        <is>
+          <t>Production reference cost per month (USD)</t>
+        </is>
+      </c>
+      <c r="B77" s="21">
+        <f>SUM(B71:B76)</f>
+        <v/>
+      </c>
+      <c r="C77" s="21">
+        <f>SUM(C71:C76)</f>
+        <v/>
+      </c>
+      <c r="D77" s="21">
+        <f>SUM(D71:D76)</f>
+        <v/>
+      </c>
+      <c r="E77" s="21">
+        <f>SUM(E71:E76)</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="inlineStr">
-        <is>
-          <t>Pre-Prod months of use per major release</t>
-        </is>
-      </c>
-      <c r="B79" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: created from a production backup for the release rehearsal and removed after the release.</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="n"/>
-      <c r="F79" s="8" t="n"/>
-      <c r="G79" s="8" t="n"/>
-      <c r="H79" s="8" t="n"/>
-      <c r="I79" s="8" t="n"/>
-      <c r="J79" s="8" t="n"/>
-      <c r="K79" s="8" t="n"/>
-      <c r="L79" s="8" t="n"/>
-      <c r="M79" s="8" t="n"/>
-      <c r="N79" s="9" t="n"/>
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>Infrastructure: non-production environment sizes and Pre-Prod use</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="n"/>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="7" t="n"/>
+      <c r="F79" s="7" t="n"/>
+      <c r="G79" s="7" t="n"/>
+      <c r="H79" s="7" t="n"/>
+      <c r="I79" s="7" t="n"/>
+      <c r="J79" s="7" t="n"/>
+      <c r="K79" s="7" t="n"/>
+      <c r="L79" s="7" t="n"/>
+      <c r="M79" s="7" t="n"/>
+      <c r="N79" s="7" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>Major releases per year (yearly hosting view only)</t>
-        </is>
-      </c>
-      <c r="B80" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>releases</t>
-        </is>
-      </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>Assumption for budgeting. Major releases are announced at least 6 months ahead (Release Notes and Roadmap); the invoice follows the actual months of use.</t>
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Basis</t>
         </is>
       </c>
       <c r="E80" s="8" t="n"/>
@@ -5365,67 +5371,89 @@
       <c r="M80" s="8" t="n"/>
       <c r="N80" s="9" t="n"/>
     </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>Non-production environment, small: cloud cost per month</t>
+        </is>
+      </c>
+      <c r="B81" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 1 container of 1 vCPU, 2 GB; PostgreSQL db.t4g.medium single-AZ, 50 GB; file store; backups 7 to 14 days. Dev in every tier; UAT of Small and Medium brokers.</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="n"/>
+      <c r="F81" s="8" t="n"/>
+      <c r="G81" s="8" t="n"/>
+      <c r="H81" s="8" t="n"/>
+      <c r="I81" s="8" t="n"/>
+      <c r="J81" s="8" t="n"/>
+      <c r="K81" s="8" t="n"/>
+      <c r="L81" s="8" t="n"/>
+      <c r="M81" s="8" t="n"/>
+      <c r="N81" s="9" t="n"/>
+    </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>Infrastructure: environment set by tier, AWS reference cost per month (USD)</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="n"/>
-      <c r="C82" s="7" t="n"/>
-      <c r="D82" s="7" t="n"/>
-      <c r="E82" s="7" t="n"/>
-      <c r="F82" s="7" t="n"/>
-      <c r="G82" s="7" t="n"/>
-      <c r="H82" s="7" t="n"/>
-      <c r="I82" s="7" t="n"/>
-      <c r="J82" s="7" t="n"/>
-      <c r="K82" s="7" t="n"/>
-      <c r="L82" s="7" t="n"/>
-      <c r="M82" s="7" t="n"/>
-      <c r="N82" s="7" t="n"/>
-    </row>
-    <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="3" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>Dev</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>SIT</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>Standing environments</t>
-        </is>
-      </c>
-      <c r="G83" s="3" t="inlineStr">
-        <is>
-          <t>Pre-Prod per month of use</t>
-        </is>
-      </c>
-      <c r="H83" s="3" t="inlineStr">
-        <is>
-          <t>Environment set and basis</t>
-        </is>
-      </c>
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>Non-production environment, medium: cloud cost per month</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 2 containers of 1 vCPU, 2 GB (the second for the UAT performance test); db.t4g.large single-AZ, 100 GB; file store; load balancer. SIT and UAT of Large and Enterprise brokers.</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="n"/>
+      <c r="F82" s="8" t="n"/>
+      <c r="G82" s="8" t="n"/>
+      <c r="H82" s="8" t="n"/>
+      <c r="I82" s="8" t="n"/>
+      <c r="J82" s="8" t="n"/>
+      <c r="K82" s="8" t="n"/>
+      <c r="L82" s="8" t="n"/>
+      <c r="M82" s="8" t="n"/>
+      <c r="N82" s="9" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>Pre-Prod cloud cost relative to Production (without the DR copy)</t>
+        </is>
+      </c>
+      <c r="B83" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: Pre-Prod is restored from a production backup and runs at production topology and size, so the rehearsal measures real timings.</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="n"/>
+      <c r="F83" s="8" t="n"/>
+      <c r="G83" s="8" t="n"/>
+      <c r="H83" s="8" t="n"/>
       <c r="I83" s="8" t="n"/>
       <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="n"/>
@@ -5434,38 +5462,28 @@
       <c r="N83" s="9" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="18">
-        <f>A28</f>
-        <v/>
-      </c>
-      <c r="B84" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C84" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="E84" s="20">
-        <f>B71</f>
-        <v/>
-      </c>
-      <c r="F84" s="24">
-        <f>SUM(B84:E84)</f>
-        <v/>
-      </c>
-      <c r="G84" s="21">
-        <f>SUM(B65:B69)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H84" s="5" t="inlineStr">
-        <is>
-          <t>Dev, UAT, Production, temporary Pre-Prod. Integration and SIT in Dev, then promoted to UAT for testing.</t>
-        </is>
-      </c>
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>Pre-Prod months of use around go-live</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: created before the cutover rehearsal and removed after hypercare (1 to 2 months). Billed per month of use.</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="n"/>
+      <c r="F84" s="8" t="n"/>
+      <c r="G84" s="8" t="n"/>
+      <c r="H84" s="8" t="n"/>
       <c r="I84" s="8" t="n"/>
       <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="n"/>
@@ -5474,38 +5492,28 @@
       <c r="N84" s="9" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="18">
-        <f>A29</f>
-        <v/>
-      </c>
-      <c r="B85" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C85" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="E85" s="20">
-        <f>C71</f>
-        <v/>
-      </c>
-      <c r="F85" s="24">
-        <f>SUM(B85:E85)</f>
-        <v/>
-      </c>
-      <c r="G85" s="21">
-        <f>SUM(C65:C69)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H85" s="5" t="inlineStr">
-        <is>
-          <t>Dev, UAT, Production, temporary Pre-Prod. As Small.</t>
-        </is>
-      </c>
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>Pre-Prod months of use per major release</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: created from a production backup for the release rehearsal and removed after the release.</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="n"/>
+      <c r="F85" s="8" t="n"/>
+      <c r="G85" s="8" t="n"/>
+      <c r="H85" s="8" t="n"/>
       <c r="I85" s="8" t="n"/>
       <c r="J85" s="8" t="n"/>
       <c r="K85" s="8" t="n"/>
@@ -5514,39 +5522,28 @@
       <c r="N85" s="9" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="18">
-        <f>A30</f>
-        <v/>
-      </c>
-      <c r="B86" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C86" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="D86" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="E86" s="20">
-        <f>D71</f>
-        <v/>
-      </c>
-      <c r="F86" s="24">
-        <f>SUM(B86:E86)</f>
-        <v/>
-      </c>
-      <c r="G86" s="21">
-        <f>SUM(D65:D69)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H86" s="5" t="inlineStr">
-        <is>
-          <t>Dev, SIT, UAT, Production with high availability, temporary Pre-Prod. SIT and UAT are separate.</t>
-        </is>
-      </c>
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Major releases per year (yearly hosting view only)</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>releases</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>Assumption for budgeting. Major releases are announced at least 6 months ahead (Release Notes and Roadmap); the invoice follows the actual months of use.</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="n"/>
+      <c r="F86" s="8" t="n"/>
+      <c r="G86" s="8" t="n"/>
+      <c r="H86" s="8" t="n"/>
       <c r="I86" s="8" t="n"/>
       <c r="J86" s="8" t="n"/>
       <c r="K86" s="8" t="n"/>
@@ -5554,86 +5551,67 @@
       <c r="M86" s="8" t="n"/>
       <c r="N86" s="9" t="n"/>
     </row>
-    <row r="87">
-      <c r="A87" s="18">
-        <f>A31</f>
-        <v/>
-      </c>
-      <c r="B87" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C87" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="D87" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="E87" s="20">
-        <f>E71</f>
-        <v/>
-      </c>
-      <c r="F87" s="24">
-        <f>SUM(B87:E87)</f>
-        <v/>
-      </c>
-      <c r="G87" s="21">
-        <f>SUM(E65:E69)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H87" s="5" t="inlineStr">
-        <is>
-          <t>As Large, with the cross-region DR copy in Production.</t>
-        </is>
-      </c>
-      <c r="I87" s="8" t="n"/>
-      <c r="J87" s="8" t="n"/>
-      <c r="K87" s="8" t="n"/>
-      <c r="L87" s="8" t="n"/>
-      <c r="M87" s="8" t="n"/>
-      <c r="N87" s="9" t="n"/>
-    </row>
     <row r="88">
-      <c r="A88" s="10" t="inlineStr">
-        <is>
-          <t>Azure cost relative to AWS</t>
-        </is>
-      </c>
-      <c r="B88" s="11" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="F88" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: comparable list prices in Southeast Asia (D4s v5 Linux about USD 158 a month, S21); +5% for managed PostgreSQL and WAF differences.</t>
-        </is>
-      </c>
-      <c r="G88" s="8" t="n"/>
-      <c r="H88" s="8" t="n"/>
-      <c r="I88" s="8" t="n"/>
-      <c r="J88" s="8" t="n"/>
-      <c r="K88" s="8" t="n"/>
-      <c r="L88" s="8" t="n"/>
-      <c r="M88" s="8" t="n"/>
-      <c r="N88" s="9" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="10" t="inlineStr">
-        <is>
-          <t>Local partner cloud cost relative to AWS</t>
-        </is>
-      </c>
-      <c r="B89" s="11" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F89" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: Philippine data-centre or partner cloud priced in PHP; lower compute and bandwidth, database run as managed VM. Confirm with a partner quotation.</t>
-        </is>
-      </c>
-      <c r="G89" s="8" t="n"/>
-      <c r="H89" s="8" t="n"/>
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>Infrastructure: environment set by tier, AWS reference cost per month (USD)</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="n"/>
+      <c r="C88" s="7" t="n"/>
+      <c r="D88" s="7" t="n"/>
+      <c r="E88" s="7" t="n"/>
+      <c r="F88" s="7" t="n"/>
+      <c r="G88" s="7" t="n"/>
+      <c r="H88" s="7" t="n"/>
+      <c r="I88" s="7" t="n"/>
+      <c r="J88" s="7" t="n"/>
+      <c r="K88" s="7" t="n"/>
+      <c r="L88" s="7" t="n"/>
+      <c r="M88" s="7" t="n"/>
+      <c r="N88" s="7" t="n"/>
+    </row>
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>SIT</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Standing environments</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Prod per month of use</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Environment set and basis</t>
+        </is>
+      </c>
       <c r="I89" s="8" t="n"/>
       <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="n"/>
@@ -5641,55 +5619,120 @@
       <c r="M89" s="8" t="n"/>
       <c r="N89" s="9" t="n"/>
     </row>
+    <row r="90">
+      <c r="A90" s="18">
+        <f>A28</f>
+        <v/>
+      </c>
+      <c r="B90" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C90" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="E90" s="20">
+        <f>B77</f>
+        <v/>
+      </c>
+      <c r="F90" s="24">
+        <f>SUM(B90:E90)</f>
+        <v/>
+      </c>
+      <c r="G90" s="21">
+        <f>SUM(B71:B75)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>Dev, UAT, Production, temporary Pre-Prod. Integration and SIT in Dev, then promoted to UAT for testing.</t>
+        </is>
+      </c>
+      <c r="I90" s="8" t="n"/>
+      <c r="J90" s="8" t="n"/>
+      <c r="K90" s="8" t="n"/>
+      <c r="L90" s="8" t="n"/>
+      <c r="M90" s="8" t="n"/>
+      <c r="N90" s="9" t="n"/>
+    </row>
     <row r="91">
-      <c r="A91" s="6" t="inlineStr">
-        <is>
-          <t>Sample quote scenarios (used by Sample Quotes)</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="n"/>
-      <c r="C91" s="7" t="n"/>
-      <c r="D91" s="7" t="n"/>
-      <c r="E91" s="7" t="n"/>
-      <c r="F91" s="7" t="n"/>
-      <c r="G91" s="7" t="n"/>
-      <c r="H91" s="7" t="n"/>
-      <c r="I91" s="7" t="n"/>
-      <c r="J91" s="7" t="n"/>
-      <c r="K91" s="7" t="n"/>
-      <c r="L91" s="7" t="n"/>
-      <c r="M91" s="7" t="n"/>
-      <c r="N91" s="7" t="n"/>
+      <c r="A91" s="18">
+        <f>A29</f>
+        <v/>
+      </c>
+      <c r="B91" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C91" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="E91" s="20">
+        <f>C77</f>
+        <v/>
+      </c>
+      <c r="F91" s="24">
+        <f>SUM(B91:E91)</f>
+        <v/>
+      </c>
+      <c r="G91" s="21">
+        <f>SUM(C71:C75)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>Dev, UAT, Production, temporary Pre-Prod. As Small.</t>
+        </is>
+      </c>
+      <c r="I91" s="8" t="n"/>
+      <c r="J91" s="8" t="n"/>
+      <c r="K91" s="8" t="n"/>
+      <c r="L91" s="8" t="n"/>
+      <c r="M91" s="8" t="n"/>
+      <c r="N91" s="9" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
-        <is>
-          <t>Example 2</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>Example 3</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr"/>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G92" s="8" t="n"/>
-      <c r="H92" s="8" t="n"/>
+      <c r="A92" s="18">
+        <f>A30</f>
+        <v/>
+      </c>
+      <c r="B92" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C92" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="D92" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="E92" s="20">
+        <f>D77</f>
+        <v/>
+      </c>
+      <c r="F92" s="24">
+        <f>SUM(B92:E92)</f>
+        <v/>
+      </c>
+      <c r="G92" s="21">
+        <f>SUM(D71:D75)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>Dev, SIT, UAT, Production with high availability, temporary Pre-Prod. SIT and UAT are separate.</t>
+        </is>
+      </c>
       <c r="I92" s="8" t="n"/>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
@@ -5698,33 +5741,39 @@
       <c r="N92" s="9" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="10" t="inlineStr">
-        <is>
-          <t>Broker profile</t>
-        </is>
-      </c>
-      <c r="B93" s="12" t="inlineStr">
-        <is>
-          <t>Small broker</t>
-        </is>
-      </c>
-      <c r="C93" s="12" t="inlineStr">
-        <is>
-          <t>Medium broker</t>
-        </is>
-      </c>
-      <c r="D93" s="12" t="inlineStr">
-        <is>
-          <t>Large broker</t>
-        </is>
-      </c>
-      <c r="F93" s="10" t="inlineStr">
-        <is>
-          <t>Label only.</t>
-        </is>
-      </c>
-      <c r="G93" s="8" t="n"/>
-      <c r="H93" s="8" t="n"/>
+      <c r="A93" s="18">
+        <f>A31</f>
+        <v/>
+      </c>
+      <c r="B93" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C93" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="D93" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="E93" s="20">
+        <f>E77</f>
+        <v/>
+      </c>
+      <c r="F93" s="24">
+        <f>SUM(B93:E93)</f>
+        <v/>
+      </c>
+      <c r="G93" s="21">
+        <f>SUM(E71:E75)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>As Large, with the cross-region DR copy in Production.</t>
+        </is>
+      </c>
       <c r="I93" s="8" t="n"/>
       <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="n"/>
@@ -5735,21 +5784,15 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>Named users</t>
-        </is>
-      </c>
-      <c r="B94" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C94" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="D94" s="14" t="n">
-        <v>180</v>
-      </c>
-      <c r="F94" s="10" t="inlineStr">
-        <is>
-          <t>Tier follows from the user count.</t>
+          <t>Azure cost relative to AWS</t>
+        </is>
+      </c>
+      <c r="B94" s="11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: comparable list prices in Southeast Asia (D4s v5 Linux about USD 158 a month, S21); +5% for managed PostgreSQL and WAF differences.</t>
         </is>
       </c>
       <c r="G94" s="8" t="n"/>
@@ -5764,21 +5807,15 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Lines of business</t>
-        </is>
-      </c>
-      <c r="B95" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C95" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="D95" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="F95" s="10" t="inlineStr">
-        <is>
-          <t>Motor, fire, marine, casualty, engineering, bonds and so on.</t>
+          <t>Local partner cloud cost relative to AWS</t>
+        </is>
+      </c>
+      <c r="B95" s="11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F95" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: Philippine data-centre or partner cloud priced in PHP; lower compute and bandwidth, database run as managed VM. Confirm with a partner quotation.</t>
         </is>
       </c>
       <c r="G95" s="8" t="n"/>
@@ -5790,94 +5827,51 @@
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="9" t="n"/>
     </row>
-    <row r="96">
-      <c r="A96" s="10" t="inlineStr">
-        <is>
-          <t>Infrastructure provider (AWS, Azure, Local partner, Customer)</t>
-        </is>
-      </c>
-      <c r="B96" s="12" t="inlineStr">
-        <is>
-          <t>AWS</t>
-        </is>
-      </c>
-      <c r="C96" s="12" t="inlineStr">
-        <is>
-          <t>Azure</t>
-        </is>
-      </c>
-      <c r="D96" s="12" t="inlineStr">
-        <is>
-          <t>Local partner</t>
-        </is>
-      </c>
-      <c r="F96" s="10" t="inlineStr">
-        <is>
-          <t>"Customer" means the broker hosts itself: no infrastructure fee.</t>
-        </is>
-      </c>
-      <c r="G96" s="8" t="n"/>
-      <c r="H96" s="8" t="n"/>
-      <c r="I96" s="8" t="n"/>
-      <c r="J96" s="8" t="n"/>
-      <c r="K96" s="8" t="n"/>
-      <c r="L96" s="8" t="n"/>
-      <c r="M96" s="8" t="n"/>
-      <c r="N96" s="9" t="n"/>
-    </row>
     <row r="97">
-      <c r="A97" s="10" t="inlineStr">
-        <is>
-          <t>24x7 Severity 1 support (Yes/No)</t>
-        </is>
-      </c>
-      <c r="B97" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C97" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D97" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F97" s="10" t="inlineStr">
-        <is>
-          <t>Optional.</t>
-        </is>
-      </c>
-      <c r="G97" s="8" t="n"/>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
-      <c r="J97" s="8" t="n"/>
-      <c r="K97" s="8" t="n"/>
-      <c r="L97" s="8" t="n"/>
-      <c r="M97" s="8" t="n"/>
-      <c r="N97" s="9" t="n"/>
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>Sample quote scenarios (used by Sample Quotes)</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="n"/>
+      <c r="C97" s="7" t="n"/>
+      <c r="D97" s="7" t="n"/>
+      <c r="E97" s="7" t="n"/>
+      <c r="F97" s="7" t="n"/>
+      <c r="G97" s="7" t="n"/>
+      <c r="H97" s="7" t="n"/>
+      <c r="I97" s="7" t="n"/>
+      <c r="J97" s="7" t="n"/>
+      <c r="K97" s="7" t="n"/>
+      <c r="L97" s="7" t="n"/>
+      <c r="M97" s="7" t="n"/>
+      <c r="N97" s="7" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="10" t="inlineStr">
-        <is>
-          <t>Extra training days</t>
-        </is>
-      </c>
-      <c r="B98" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C98" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D98" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F98" s="10" t="inlineStr">
-        <is>
-          <t>Beyond the days included for the tier.</t>
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Example 1</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Example 2</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Example 3</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr"/>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G98" s="8" t="n"/>
@@ -5892,21 +5886,27 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>Extra legacy data sources to migrate</t>
-        </is>
-      </c>
-      <c r="B99" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C99" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D99" s="14" t="n">
-        <v>2</v>
+          <t>Broker profile</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>Small broker</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>Medium broker</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr">
+        <is>
+          <t>Large broker</t>
+        </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>Beyond the standard templates.</t>
+          <t>Label only.</t>
         </is>
       </c>
       <c r="G99" s="8" t="n"/>
@@ -5921,21 +5921,21 @@
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>Additional standard integrations</t>
+          <t>Named users</t>
         </is>
       </c>
       <c r="B100" s="14" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C100" s="14" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D100" s="14" t="n">
-        <v>2</v>
+        <v>180</v>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>One-time.</t>
+          <t>Tier follows from the user count.</t>
         </is>
       </c>
       <c r="G100" s="8" t="n"/>
@@ -5947,82 +5947,274 @@
       <c r="M100" s="8" t="n"/>
       <c r="N100" s="9" t="n"/>
     </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>Lines of business</t>
+        </is>
+      </c>
+      <c r="B101" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C101" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D101" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="F101" s="10" t="inlineStr">
+        <is>
+          <t>Motor, fire, marine, casualty, engineering, bonds and so on.</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="n"/>
+      <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="n"/>
+      <c r="J101" s="8" t="n"/>
+      <c r="K101" s="8" t="n"/>
+      <c r="L101" s="8" t="n"/>
+      <c r="M101" s="8" t="n"/>
+      <c r="N101" s="9" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Infrastructure provider (AWS, Azure, Local partner, Customer)</t>
+        </is>
+      </c>
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr">
+        <is>
+          <t>Local partner</t>
+        </is>
+      </c>
+      <c r="F102" s="10" t="inlineStr">
+        <is>
+          <t>"Customer" means the broker hosts itself: no infrastructure fee.</t>
+        </is>
+      </c>
+      <c r="G102" s="8" t="n"/>
+      <c r="H102" s="8" t="n"/>
+      <c r="I102" s="8" t="n"/>
+      <c r="J102" s="8" t="n"/>
+      <c r="K102" s="8" t="n"/>
+      <c r="L102" s="8" t="n"/>
+      <c r="M102" s="8" t="n"/>
+      <c r="N102" s="9" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>24x7 Severity 1 support (Yes/No)</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>Optional.</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="n"/>
+      <c r="H103" s="8" t="n"/>
+      <c r="I103" s="8" t="n"/>
+      <c r="J103" s="8" t="n"/>
+      <c r="K103" s="8" t="n"/>
+      <c r="L103" s="8" t="n"/>
+      <c r="M103" s="8" t="n"/>
+      <c r="N103" s="9" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="inlineStr">
+        <is>
+          <t>Extra training days</t>
+        </is>
+      </c>
+      <c r="B104" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D104" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" s="10" t="inlineStr">
+        <is>
+          <t>Beyond the days included for the tier.</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="n"/>
+      <c r="H104" s="8" t="n"/>
+      <c r="I104" s="8" t="n"/>
+      <c r="J104" s="8" t="n"/>
+      <c r="K104" s="8" t="n"/>
+      <c r="L104" s="8" t="n"/>
+      <c r="M104" s="8" t="n"/>
+      <c r="N104" s="9" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>Extra legacy data sources to migrate</t>
+        </is>
+      </c>
+      <c r="B105" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C105" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>Beyond the standard templates.</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="n"/>
+      <c r="H105" s="8" t="n"/>
+      <c r="I105" s="8" t="n"/>
+      <c r="J105" s="8" t="n"/>
+      <c r="K105" s="8" t="n"/>
+      <c r="L105" s="8" t="n"/>
+      <c r="M105" s="8" t="n"/>
+      <c r="N105" s="9" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>Additional standard integrations</t>
+        </is>
+      </c>
+      <c r="B106" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F106" s="10" t="inlineStr">
+        <is>
+          <t>One-time.</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="n"/>
+      <c r="H106" s="8" t="n"/>
+      <c r="I106" s="8" t="n"/>
+      <c r="J106" s="8" t="n"/>
+      <c r="K106" s="8" t="n"/>
+      <c r="L106" s="8" t="n"/>
+      <c r="M106" s="8" t="n"/>
+      <c r="N106" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="68">
+  <mergeCells count="74">
     <mergeCell ref="E36:N36"/>
     <mergeCell ref="D59:N59"/>
-    <mergeCell ref="D79:N79"/>
     <mergeCell ref="D50:N50"/>
-    <mergeCell ref="H84:N84"/>
+    <mergeCell ref="F104:N104"/>
     <mergeCell ref="D60:N60"/>
+    <mergeCell ref="F76:N76"/>
     <mergeCell ref="F95:N95"/>
     <mergeCell ref="D19:N19"/>
+    <mergeCell ref="D63:N63"/>
     <mergeCell ref="F94:N94"/>
     <mergeCell ref="D10:N10"/>
-    <mergeCell ref="H87:N87"/>
+    <mergeCell ref="F101:N101"/>
     <mergeCell ref="F70:N70"/>
-    <mergeCell ref="F97:N97"/>
-    <mergeCell ref="F66:N66"/>
+    <mergeCell ref="D81:N81"/>
     <mergeCell ref="D46:N46"/>
-    <mergeCell ref="H86:N86"/>
+    <mergeCell ref="D84:N84"/>
+    <mergeCell ref="F75:N75"/>
+    <mergeCell ref="F106:N106"/>
     <mergeCell ref="D80:N80"/>
     <mergeCell ref="E41:N41"/>
+    <mergeCell ref="D65:N65"/>
+    <mergeCell ref="D45:N45"/>
     <mergeCell ref="F100:N100"/>
-    <mergeCell ref="D45:N45"/>
+    <mergeCell ref="F72:N72"/>
     <mergeCell ref="E37:N37"/>
     <mergeCell ref="D6:N6"/>
     <mergeCell ref="D52:N52"/>
-    <mergeCell ref="D77:N77"/>
+    <mergeCell ref="H92:N92"/>
+    <mergeCell ref="D86:N86"/>
     <mergeCell ref="D11:N11"/>
     <mergeCell ref="D49:N49"/>
     <mergeCell ref="D57:N57"/>
-    <mergeCell ref="F93:N93"/>
-    <mergeCell ref="F96:N96"/>
+    <mergeCell ref="H91:N91"/>
+    <mergeCell ref="F102:N102"/>
+    <mergeCell ref="F71:N71"/>
     <mergeCell ref="D13:N13"/>
-    <mergeCell ref="F67:N67"/>
-    <mergeCell ref="D76:N76"/>
+    <mergeCell ref="F105:N105"/>
     <mergeCell ref="E42:N42"/>
     <mergeCell ref="D48:N48"/>
     <mergeCell ref="D17:N17"/>
     <mergeCell ref="D61:N61"/>
-    <mergeCell ref="F92:N92"/>
-    <mergeCell ref="D75:N75"/>
     <mergeCell ref="D53:N53"/>
+    <mergeCell ref="D66:N66"/>
+    <mergeCell ref="H93:N93"/>
     <mergeCell ref="E39:N39"/>
     <mergeCell ref="D16:N16"/>
     <mergeCell ref="D47:N47"/>
     <mergeCell ref="F98:N98"/>
     <mergeCell ref="D7:N7"/>
-    <mergeCell ref="D78:N78"/>
-    <mergeCell ref="H83:N83"/>
     <mergeCell ref="E35:N35"/>
-    <mergeCell ref="F88:N88"/>
-    <mergeCell ref="F64:N64"/>
     <mergeCell ref="E38:N38"/>
+    <mergeCell ref="D62:N62"/>
     <mergeCell ref="A32:N32"/>
+    <mergeCell ref="F73:N73"/>
     <mergeCell ref="D18:N18"/>
     <mergeCell ref="D56:N56"/>
-    <mergeCell ref="F69:N69"/>
+    <mergeCell ref="H89:N89"/>
     <mergeCell ref="D9:N9"/>
     <mergeCell ref="D12:N12"/>
     <mergeCell ref="D58:N58"/>
     <mergeCell ref="D8:N8"/>
-    <mergeCell ref="F68:N68"/>
-    <mergeCell ref="F65:N65"/>
-    <mergeCell ref="D74:N74"/>
-    <mergeCell ref="H85:N85"/>
+    <mergeCell ref="D83:N83"/>
+    <mergeCell ref="F103:N103"/>
+    <mergeCell ref="D64:N64"/>
+    <mergeCell ref="D15:N15"/>
+    <mergeCell ref="D82:N82"/>
     <mergeCell ref="F99:N99"/>
-    <mergeCell ref="D15:N15"/>
-    <mergeCell ref="F89:N89"/>
+    <mergeCell ref="D67:N67"/>
     <mergeCell ref="D5:N5"/>
     <mergeCell ref="D51:N51"/>
+    <mergeCell ref="F74:N74"/>
     <mergeCell ref="D14:N14"/>
+    <mergeCell ref="D85:N85"/>
+    <mergeCell ref="H90:N90"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B96:D96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B102:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"AWS,Azure,Local partner,Customer"</formula1>
     </dataValidation>
-    <dataValidation sqref="B97:D97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B103:D103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10243,19 +10435,19 @@
         </is>
       </c>
       <c r="D5" s="27">
-        <f>ROUND(Inputs!B84*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B90*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E5" s="27">
-        <f>ROUND(Inputs!C84*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C90*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F5" s="27">
-        <f>ROUND(Inputs!D84*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D90*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G5" s="27">
-        <f>ROUND(Inputs!E84*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E90*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H5" s="24">
@@ -10263,7 +10455,7 @@
         <v/>
       </c>
       <c r="I5" s="24">
-        <f>ROUND(Inputs!G84*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G90*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J5" s="20">
@@ -10300,19 +10492,19 @@
         </is>
       </c>
       <c r="D6" s="27">
-        <f>ROUND(Inputs!B85*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B91*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E6" s="27">
-        <f>ROUND(Inputs!C85*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C91*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F6" s="27">
-        <f>ROUND(Inputs!D85*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D91*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G6" s="27">
-        <f>ROUND(Inputs!E85*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E91*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H6" s="24">
@@ -10320,7 +10512,7 @@
         <v/>
       </c>
       <c r="I6" s="24">
-        <f>ROUND(Inputs!G85*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G91*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J6" s="20">
@@ -10353,19 +10545,19 @@
         </is>
       </c>
       <c r="D7" s="27">
-        <f>ROUND(Inputs!B86*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B92*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E7" s="27">
-        <f>ROUND(Inputs!C86*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C92*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F7" s="27">
-        <f>ROUND(Inputs!D86*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D92*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G7" s="27">
-        <f>ROUND(Inputs!E86*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E92*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H7" s="24">
@@ -10373,7 +10565,7 @@
         <v/>
       </c>
       <c r="I7" s="24">
-        <f>ROUND(Inputs!G86*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G92*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J7" s="20">
@@ -10406,19 +10598,19 @@
         </is>
       </c>
       <c r="D8" s="27">
-        <f>ROUND(Inputs!B87*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B93*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E8" s="27">
-        <f>ROUND(Inputs!C87*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C93*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F8" s="27">
-        <f>ROUND(Inputs!D87*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D93*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G8" s="27">
-        <f>ROUND(Inputs!E87*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E93*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H8" s="24">
@@ -10426,7 +10618,7 @@
         <v/>
       </c>
       <c r="I8" s="24">
-        <f>ROUND(Inputs!G87*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G93*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J8" s="20">
@@ -10459,19 +10651,19 @@
         </is>
       </c>
       <c r="D9" s="27">
-        <f>ROUND(Inputs!B84*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E9" s="27">
-        <f>ROUND(Inputs!C84*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F9" s="27">
-        <f>ROUND(Inputs!D84*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G9" s="27">
-        <f>ROUND(Inputs!E84*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H9" s="24">
@@ -10479,7 +10671,7 @@
         <v/>
       </c>
       <c r="I9" s="24">
-        <f>ROUND(Inputs!G84*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J9" s="20">
@@ -10516,19 +10708,19 @@
         </is>
       </c>
       <c r="D10" s="27">
-        <f>ROUND(Inputs!B85*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>ROUND(Inputs!C85*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>ROUND(Inputs!D85*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>ROUND(Inputs!E85*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H10" s="24">
@@ -10536,7 +10728,7 @@
         <v/>
       </c>
       <c r="I10" s="24">
-        <f>ROUND(Inputs!G85*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J10" s="20">
@@ -10569,19 +10761,19 @@
         </is>
       </c>
       <c r="D11" s="27">
-        <f>ROUND(Inputs!B86*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>ROUND(Inputs!C86*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>ROUND(Inputs!D86*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G11" s="27">
-        <f>ROUND(Inputs!E86*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H11" s="24">
@@ -10589,7 +10781,7 @@
         <v/>
       </c>
       <c r="I11" s="24">
-        <f>ROUND(Inputs!G86*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J11" s="20">
@@ -10622,19 +10814,19 @@
         </is>
       </c>
       <c r="D12" s="27">
-        <f>ROUND(Inputs!B87*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E12" s="27">
-        <f>ROUND(Inputs!C87*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F12" s="27">
-        <f>ROUND(Inputs!D87*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G12" s="27">
-        <f>ROUND(Inputs!E87*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H12" s="24">
@@ -10642,7 +10834,7 @@
         <v/>
       </c>
       <c r="I12" s="24">
-        <f>ROUND(Inputs!G87*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J12" s="20">
@@ -10675,19 +10867,19 @@
         </is>
       </c>
       <c r="D13" s="27">
-        <f>ROUND(Inputs!B84*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E13" s="27">
-        <f>ROUND(Inputs!C84*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F13" s="27">
-        <f>ROUND(Inputs!D84*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G13" s="27">
-        <f>ROUND(Inputs!E84*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H13" s="24">
@@ -10695,7 +10887,7 @@
         <v/>
       </c>
       <c r="I13" s="24">
-        <f>ROUND(Inputs!G84*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J13" s="20">
@@ -10732,19 +10924,19 @@
         </is>
       </c>
       <c r="D14" s="27">
-        <f>ROUND(Inputs!B85*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E14" s="27">
-        <f>ROUND(Inputs!C85*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F14" s="27">
-        <f>ROUND(Inputs!D85*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G14" s="27">
-        <f>ROUND(Inputs!E85*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H14" s="24">
@@ -10752,7 +10944,7 @@
         <v/>
       </c>
       <c r="I14" s="24">
-        <f>ROUND(Inputs!G85*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J14" s="20">
@@ -10785,19 +10977,19 @@
         </is>
       </c>
       <c r="D15" s="27">
-        <f>ROUND(Inputs!B86*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E15" s="27">
-        <f>ROUND(Inputs!C86*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F15" s="27">
-        <f>ROUND(Inputs!D86*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G15" s="27">
-        <f>ROUND(Inputs!E86*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H15" s="24">
@@ -10805,7 +10997,7 @@
         <v/>
       </c>
       <c r="I15" s="24">
-        <f>ROUND(Inputs!G86*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J15" s="20">
@@ -10838,19 +11030,19 @@
         </is>
       </c>
       <c r="D16" s="27">
-        <f>ROUND(Inputs!B87*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E16" s="27">
-        <f>ROUND(Inputs!C87*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F16" s="27">
-        <f>ROUND(Inputs!D87*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G16" s="27">
-        <f>ROUND(Inputs!E87*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H16" s="24">
@@ -10858,7 +11050,7 @@
         <v/>
       </c>
       <c r="I16" s="24">
-        <f>ROUND(Inputs!G87*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J16" s="20">
@@ -11921,7 +12113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -12175,16 +12367,16 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Additional line of business after go-live</t>
+          <t>Connector go-live with a partner</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>per line</t>
+          <t>per connector</t>
         </is>
       </c>
       <c r="C12" s="34">
-        <f>ROUND(Days_per_LOB*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(Conn_Golive_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D12" s="20">
@@ -12192,28 +12384,28 @@
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>Days_per_LOB</f>
+        <f>Conn_Golive_Days</f>
         <v/>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Product set-up, rating and tax lines, templates, testing.</t>
+          <t>To confirm by management. A delivered connector (SMS gateway, CTPL provider, one insurer, one bank file layout, BIR EIS) taken live; the partner certifies its own side.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>New report or document template</t>
+          <t>Activation of the AML/CFT toolkit</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>per item (typical)</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C13" s="34">
-        <f>ROUND(Report_Days*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(AML_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D13" s="20">
@@ -12221,171 +12413,353 @@
         <v/>
       </c>
       <c r="E13" s="25">
-        <f>Report_Days</f>
+        <f>AML_Act_Days</f>
         <v/>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Small CR band; firm price after the impact note.</t>
+          <t>To confirm by management. The toolkit is included in the software; this is the set-up effort. The compliance officer confirms the settings and loads the lists.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>On-site day (Metro Manila)</t>
+          <t>Activation of the IC compliance registers</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>per consultant day</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C14" s="34">
-        <f>Rate_Onsite</f>
+        <f>ROUND(IC_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D14" s="20">
         <f>C14/FX</f>
         <v/>
       </c>
-      <c r="E14" s="25" t="inlineStr"/>
+      <c r="E14" s="25">
+        <f>IC_Act_Days</f>
+        <v/>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Outside Metro Manila: travel, lodging and meals at cost.</t>
+          <t>To confirm by management. Registers included in the software; this is the set-up effort.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A28&amp;" tier"</f>
-        <v/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Activation of the BIR pack</t>
+        </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C15" s="34">
-        <f>Inputs!L28</f>
+        <f>ROUND(BIR_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D15" s="20">
         <f>C15/FX</f>
         <v/>
       </c>
+      <c r="E15" s="25">
+        <f>BIR_Act_Days</f>
+        <v/>
+      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Standard support is business hours (Monday to Friday, 08:00 to 18:00 Philippine time, excluding holidays). This adds round-the-clock response to Severity 1 incidents (production down or a core process stopped for all users).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A29&amp;" tier"</f>
-        <v/>
+          <t>To confirm by management. BIR forms, EOPT invoices, EIS and CAS pack included in the software; the tax adviser confirms the treatment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Dealer programme set-up</t>
+        </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>per programme</t>
         </is>
       </c>
       <c r="C16" s="34">
-        <f>Inputs!L29</f>
+        <f>ROUND(Dealer_Prog_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D16" s="20">
         <f>C16/FX</f>
         <v/>
       </c>
-      <c r="F16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A30&amp;" tier"</f>
-        <v/>
+      <c r="E16" s="25">
+        <f>Dealer_Prog_Days</f>
+        <v/>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>To confirm by management. Dealer programmes are included in the software; this is the set-up of one programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Client brand pack</t>
+        </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>per pack</t>
         </is>
       </c>
       <c r="C17" s="34">
-        <f>Inputs!L30</f>
+        <f>ROUND(Brand_Pack_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D17" s="20">
         <f>C17/FX</f>
         <v/>
       </c>
-      <c r="F17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A31&amp;" tier"</f>
-        <v/>
+      <c r="E17" s="25">
+        <f>Brand_Pack_Days</f>
+        <v/>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>To confirm by management. Branding is included in the software; a pack carrying third-party marks needs the owner's written permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Additional line of business after go-live</t>
+        </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>per line</t>
         </is>
       </c>
       <c r="C18" s="34">
-        <f>Inputs!L31</f>
+        <f>ROUND(Days_per_LOB*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D18" s="20">
         <f>C18/FX</f>
         <v/>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="E18" s="25">
+        <f>Days_per_LOB</f>
+        <v/>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Product set-up, rating and tax lines, templates, testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>New report or document template</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>per item (typical)</t>
+        </is>
+      </c>
+      <c r="C19" s="34">
+        <f>ROUND(Report_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D19" s="20">
+        <f>C19/FX</f>
+        <v/>
+      </c>
+      <c r="E19" s="25">
+        <f>Report_Days</f>
+        <v/>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Small CR band; firm price after the impact note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>On-site day (Metro Manila)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>per consultant day</t>
+        </is>
+      </c>
+      <c r="C20" s="34">
+        <f>Rate_Onsite</f>
+        <v/>
+      </c>
+      <c r="D20" s="20">
+        <f>C20/FX</f>
+        <v/>
+      </c>
+      <c r="E20" s="25" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Outside Metro Manila: travel, lodging and meals at cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A28&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C21" s="34">
+        <f>Inputs!L28</f>
+        <v/>
+      </c>
+      <c r="D21" s="20">
+        <f>C21/FX</f>
+        <v/>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Standard support is business hours (Monday to Friday, 08:00 to 18:00 Philippine time, excluding holidays). This adds round-the-clock response to Severity 1 incidents (production down or a core process stopped for all users).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A29&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C22" s="34">
+        <f>Inputs!L29</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>C22/FX</f>
+        <v/>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A30&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C23" s="34">
+        <f>Inputs!L30</f>
+        <v/>
+      </c>
+      <c r="D23" s="20">
+        <f>C23/FX</f>
+        <v/>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A31&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C24" s="34">
+        <f>Inputs!L31</f>
+        <v/>
+      </c>
+      <c r="D24" s="20">
+        <f>C24/FX</f>
+        <v/>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Included in the standard implementation (no extra charge)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Configuration of the company, branches, users and roles, insurers, commission rates, chart of accounts, banks and the included lines of business.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>Data load using the standard upload templates (about 50 templates in docs/package/05_Delivery/Upload_Templates), with the broker supplying clean data.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="26" t="inlineStr">
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>Training days included for the tier (train-the-trainer), UAT support, go-live support and 4 weeks of hypercare.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>Set-up of the environment set of the tier (Dev, UAT and Production; SIT as well for Large and Enterprise) and of Pre-Prod for the go-live rehearsal; hosting is billed separately. Deployment guidance when the broker hosts.</t>
         </is>
       </c>
     </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>Every module is included in the software price, including the AML/CFT toolkit, the IC compliance registers, the BIR pack, the integration framework with its connectors, dealer programmes and branding. Their activation and each connector go-live are the optional lines above (to confirm by management).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:F23"/>
+  <mergeCells count="5">
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <printOptions gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12436,7 +12810,7 @@
     </row>
     <row r="4">
       <c r="A4" s="6">
-        <f>"Example 1: "&amp;Inputs!$B$93&amp;", "&amp;Inputs!$B$94&amp;" users, "&amp;Inputs!$B$95&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$B$96</f>
+        <f>"Example 1: "&amp;Inputs!$B$99&amp;", "&amp;Inputs!$B$100&amp;" users, "&amp;Inputs!$B$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$B$102</f>
         <v/>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -12503,7 +12877,7 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$B$95-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$B$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C7" s="20" t="n">
@@ -12534,7 +12908,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>MAX(0,MIN(Inputs!$B$94,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$B$94,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$B$94,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$B$94,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$B$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$B$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$B$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$B$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C8" s="20" t="n">
@@ -12668,27 +13042,27 @@
     </row>
     <row r="13">
       <c r="A13" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G13" s="34">
@@ -12744,27 +13118,27 @@
     </row>
     <row r="16">
       <c r="A16" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$B$96</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$B$102</f>
         <v/>
       </c>
       <c r="B16" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$B$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G16" s="34">
@@ -12783,23 +13157,23 @@
         </is>
       </c>
       <c r="B17" s="20">
-        <f>IF(Inputs!$B$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>IF(Inputs!$B$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>IF(Inputs!$B$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E17" s="20">
-        <f>IF(Inputs!$B$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F17" s="20">
-        <f>IF(Inputs!$B$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G17" s="34">
@@ -12818,7 +13192,7 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <f>Inputs!$B$98*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$B$99+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$B$100</f>
+        <f>Inputs!$B$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$B$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$B$106</f>
         <v/>
       </c>
       <c r="C18" s="20" t="n">
@@ -13060,7 +13434,7 @@
     </row>
     <row r="27">
       <c r="A27" s="6">
-        <f>"Example 2: "&amp;Inputs!$C$93&amp;", "&amp;Inputs!$C$94&amp;" users, "&amp;Inputs!$C$95&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$C$96</f>
+        <f>"Example 2: "&amp;Inputs!$C$99&amp;", "&amp;Inputs!$C$100&amp;" users, "&amp;Inputs!$C$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$C$102</f>
         <v/>
       </c>
       <c r="B27" s="7" t="n"/>
@@ -13127,7 +13501,7 @@
         </is>
       </c>
       <c r="B30" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$C$95-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$C$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C30" s="20" t="n">
@@ -13158,7 +13532,7 @@
         </is>
       </c>
       <c r="B31" s="20">
-        <f>MAX(0,MIN(Inputs!$C$94,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$C$94,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$C$94,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$C$94,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$C$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$C$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$C$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$C$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C31" s="20" t="n">
@@ -13292,27 +13666,27 @@
     </row>
     <row r="36">
       <c r="A36" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G36" s="34">
@@ -13368,27 +13742,27 @@
     </row>
     <row r="39">
       <c r="A39" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$C$96</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$C$102</f>
         <v/>
       </c>
       <c r="B39" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$C$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G39" s="34">
@@ -13407,23 +13781,23 @@
         </is>
       </c>
       <c r="B40" s="20">
-        <f>IF(Inputs!$C$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C40" s="20">
-        <f>IF(Inputs!$C$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D40" s="20">
-        <f>IF(Inputs!$C$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E40" s="20">
-        <f>IF(Inputs!$C$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F40" s="20">
-        <f>IF(Inputs!$C$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G40" s="34">
@@ -13442,7 +13816,7 @@
         </is>
       </c>
       <c r="B41" s="20">
-        <f>Inputs!$C$98*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$C$99+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$C$100</f>
+        <f>Inputs!$C$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$C$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$C$106</f>
         <v/>
       </c>
       <c r="C41" s="20" t="n">
@@ -13684,7 +14058,7 @@
     </row>
     <row r="50">
       <c r="A50" s="6">
-        <f>"Example 3: "&amp;Inputs!$D$93&amp;", "&amp;Inputs!$D$94&amp;" users, "&amp;Inputs!$D$95&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$D$96</f>
+        <f>"Example 3: "&amp;Inputs!$D$99&amp;", "&amp;Inputs!$D$100&amp;" users, "&amp;Inputs!$D$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$D$102</f>
         <v/>
       </c>
       <c r="B50" s="7" t="n"/>
@@ -13751,7 +14125,7 @@
         </is>
       </c>
       <c r="B53" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$D$95-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$D$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C53" s="20" t="n">
@@ -13782,7 +14156,7 @@
         </is>
       </c>
       <c r="B54" s="20">
-        <f>MAX(0,MIN(Inputs!$D$94,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$D$94,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$D$94,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$D$94,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$D$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$D$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$D$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$D$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C54" s="20" t="n">
@@ -13916,27 +14290,27 @@
     </row>
     <row r="59">
       <c r="A59" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$94,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G59" s="34">
@@ -13992,27 +14366,27 @@
     </row>
     <row r="62">
       <c r="A62" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$D$96</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$D$102</f>
         <v/>
       </c>
       <c r="B62" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$D$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$96,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G62" s="34">
@@ -14031,23 +14405,23 @@
         </is>
       </c>
       <c r="B63" s="20">
-        <f>IF(Inputs!$D$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C63" s="20">
-        <f>IF(Inputs!$D$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D63" s="20">
-        <f>IF(Inputs!$D$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E63" s="20">
-        <f>IF(Inputs!$D$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F63" s="20">
-        <f>IF(Inputs!$D$97="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$94,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G63" s="34">
@@ -14066,7 +14440,7 @@
         </is>
       </c>
       <c r="B64" s="20">
-        <f>Inputs!$D$98*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$D$99+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$D$100</f>
+        <f>Inputs!$D$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$D$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$D$106</f>
         <v/>
       </c>
       <c r="C64" s="20" t="n">

</xml_diff>

<commit_message>
Commercial and contract documents: optional services confirmed by management on 04 October 2026 (six activation and connector go-live lines are standard optional services; ten regulator and partner items added as optional modules and partner services at man-days x PHP 16,100 rounded to PHP 10,000; package totals unchanged); Rate Card 1.1.1, Commercial Proposal Note 1.1.1, Negotiation Playbook 1.0.1, Service Catalogue and Rate Annex 1.0.1, OOTB Strategy 1.1.2 (decisions 11 and 12 taken), PH Fit Assessment 1.1.2, FAQ 1.1.2; pricing workbook and price book rebuilt
</commit_message>
<xml_diff>
--- a/docs/package/02_Commercials/BrokerVerse_Commercials_and_Pricing.xlsx
+++ b/docs/package/02_Commercials/BrokerVerse_Commercials_and_Pricing.xlsx
@@ -62,14 +62,24 @@
     <definedName name="BIR_Act_Days">Inputs!$B$65</definedName>
     <definedName name="Dealer_Prog_Days">Inputs!$B$66</definedName>
     <definedName name="Brand_Pack_Days">Inputs!$B$67</definedName>
-    <definedName name="NP_Small_USD">Inputs!$B$81</definedName>
-    <definedName name="NP_Med_USD">Inputs!$B$82</definedName>
-    <definedName name="PreProd_Factor">Inputs!$B$83</definedName>
-    <definedName name="PreProd_GoLive_Months">Inputs!$B$84</definedName>
-    <definedName name="PreProd_Rel_Months">Inputs!$B$85</definedName>
-    <definedName name="Major_Rel_Year">Inputs!$B$86</definedName>
-    <definedName name="Azure_Factor">Inputs!$B$94</definedName>
-    <definedName name="Local_Factor">Inputs!$B$95</definedName>
+    <definedName name="AMLC_Val_Days">Inputs!$B$68</definedName>
+    <definedName name="IC_Form_Days">Inputs!$B$69</definedName>
+    <definedName name="EOPT_Rev_Days">Inputs!$B$70</definedName>
+    <definedName name="CAS_Reg_Days">Inputs!$B$71</definedName>
+    <definedName name="EIS_Enrol_Days">Inputs!$B$72</definedName>
+    <definedName name="CTPL_Cert_Days">Inputs!$B$73</definedName>
+    <definedName name="Insurer_Onb_Days">Inputs!$B$74</definedName>
+    <definedName name="Bank_Cert_Days">Inputs!$B$75</definedName>
+    <definedName name="SMS_Act_Days">Inputs!$B$76</definedName>
+    <definedName name="Screen_Prov_Days">Inputs!$B$77</definedName>
+    <definedName name="NP_Small_USD">Inputs!$B$91</definedName>
+    <definedName name="NP_Med_USD">Inputs!$B$92</definedName>
+    <definedName name="PreProd_Factor">Inputs!$B$93</definedName>
+    <definedName name="PreProd_GoLive_Months">Inputs!$B$94</definedName>
+    <definedName name="PreProd_Rel_Months">Inputs!$B$95</definedName>
+    <definedName name="Major_Rel_Year">Inputs!$B$96</definedName>
+    <definedName name="Azure_Factor">Inputs!$B$104</definedName>
+    <definedName name="Local_Factor">Inputs!$B$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -661,7 +671,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>iorta TechNXT. Prepared 03 October 2026. Prices in PHP, exclusive of 12% VAT. For discussion with prospective broker customers.</t>
+          <t>iorta TechNXT. Prepared 03 October 2026, revised 04 October 2026 (optional modules and partner services confirmed). Prices in PHP, exclusive of 12% VAT. For discussion with prospective broker customers.</t>
         </is>
       </c>
     </row>
@@ -3222,7 +3232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4867,7 +4877,7 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Go-live of a delivered connector with one partner (to confirm by management)</t>
+          <t>Go-live of a delivered connector with one partner</t>
         </is>
       </c>
       <c r="B62" s="14" t="n">
@@ -4880,7 +4890,7 @@
       </c>
       <c r="D62" s="15" t="inlineStr">
         <is>
-          <t>Assumption: SMS gateway, CTPL provider, one insurer API mapping, one bank file layout or the BIR EIS: configuration, credentials check, live test, support of the partner acceptance. To confirm by management.</t>
+          <t>Estimate: SMS gateway, CTPL provider, one insurer API mapping, one bank file layout or the BIR EIS: configuration, credentials check, live test, support of the partner acceptance. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E62" s="8" t="n"/>
@@ -4897,7 +4907,7 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Activation of the AML/CFT toolkit (to confirm by management)</t>
+          <t>Activation of the AML/CFT toolkit</t>
         </is>
       </c>
       <c r="B63" s="14" t="n">
@@ -4910,7 +4920,7 @@
       </c>
       <c r="D63" s="15" t="inlineStr">
         <is>
-          <t>Assumption: risk factors and rules workshop with the compliance officer, settings, first list loads, provider set-up, AMLC test file. To confirm by management.</t>
+          <t>Estimate: risk factors and rules workshop with the compliance officer, settings, first list loads, provider set-up, AMLC test file. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E63" s="8" t="n"/>
@@ -4927,7 +4937,7 @@
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>Activation of the IC compliance registers (to confirm by management)</t>
+          <t>Activation of the IC compliance registers</t>
         </is>
       </c>
       <c r="B64" s="14" t="n">
@@ -4940,7 +4950,7 @@
       </c>
       <c r="D64" s="15" t="inlineStr">
         <is>
-          <t>Assumption: licence and fit and proper register load, insurer certificates, complaints and breach settings, IC statement account mapping to the broker chart. To confirm by management.</t>
+          <t>Estimate: licence and fit and proper register load, insurer certificates, complaints and breach settings, IC statement account mapping to the broker chart. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E64" s="8" t="n"/>
@@ -4957,7 +4967,7 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Activation of the BIR pack (to confirm by management)</t>
+          <t>Activation of the BIR pack</t>
         </is>
       </c>
       <c r="B65" s="14" t="n">
@@ -4970,7 +4980,7 @@
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>Assumption: BIR and EOPT invoice settings with the tax adviser, ATC mapping, DAT file dry run, CAS books pack. To confirm by management.</t>
+          <t>Estimate: BIR and EOPT invoice settings with the tax adviser, ATC mapping, DAT file dry run, CAS books pack. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E65" s="8" t="n"/>
@@ -4987,7 +4997,7 @@
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Set-up of one dealer programme (to confirm by management)</t>
+          <t>Set-up of one dealer programme</t>
         </is>
       </c>
       <c r="B66" s="14" t="n">
@@ -5000,7 +5010,7 @@
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>Assumption: channels, rates, subsidy, bank letter and the first upload. To confirm by management.</t>
+          <t>Estimate: channels, rates, subsidy, bank letter and the first upload. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E66" s="8" t="n"/>
@@ -5017,7 +5027,7 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Client brand pack (to confirm by management)</t>
+          <t>Client brand pack</t>
         </is>
       </c>
       <c r="B67" s="14" t="n">
@@ -5030,7 +5040,7 @@
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>Assumption: theme, sign-in picture, document and e-mail branding, e-signature mapping, exported pack. To confirm by management.</t>
+          <t>Estimate: theme, sign-in picture, document and e-mail branding, e-signature mapping, exported pack. Optional service confirmed by management on 04 October 2026.</t>
         </is>
       </c>
       <c r="E67" s="8" t="n"/>
@@ -5044,57 +5054,87 @@
       <c r="M67" s="8" t="n"/>
       <c r="N67" s="9" t="n"/>
     </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>AMLC reporting file validation and portal test</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: CTR and STR layout, institution and transaction codes confirmed with the AMLC, test file accepted in the AMLC portal. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
+      <c r="L68" s="8" t="n"/>
+      <c r="M68" s="8" t="n"/>
+      <c r="N68" s="9" t="n"/>
+    </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>Infrastructure: AWS reference cost per month of the Production environment (USD)</t>
-        </is>
-      </c>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="n"/>
-      <c r="E69" s="7" t="n"/>
-      <c r="F69" s="7" t="n"/>
-      <c r="G69" s="7" t="n"/>
-      <c r="H69" s="7" t="n"/>
-      <c r="I69" s="7" t="n"/>
-      <c r="J69" s="7" t="n"/>
-      <c r="K69" s="7" t="n"/>
-      <c r="L69" s="7" t="n"/>
-      <c r="M69" s="7" t="n"/>
-      <c r="N69" s="7" t="n"/>
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>IC annual statement form alignment</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: the accountant working paper mapped to the IC form set in force for the year. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+      <c r="J69" s="8" t="n"/>
+      <c r="K69" s="8" t="n"/>
+      <c r="L69" s="8" t="n"/>
+      <c r="M69" s="8" t="n"/>
+      <c r="N69" s="9" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>EOPT invoicing review with the broker tax adviser</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: registered invoice documents, supplementary wording, VAT treatment, ATP or CAS. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="n"/>
+      <c r="F70" s="8" t="n"/>
       <c r="G70" s="8" t="n"/>
       <c r="H70" s="8" t="n"/>
       <c r="I70" s="8" t="n"/>
@@ -5107,26 +5147,24 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>Application containers (API, web, scheduler)</t>
-        </is>
-      </c>
-      <c r="B71" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="C71" s="16" t="n">
-        <v>135</v>
-      </c>
-      <c r="D71" s="16" t="n">
-        <v>180</v>
-      </c>
-      <c r="E71" s="16" t="n">
-        <v>360</v>
-      </c>
-      <c r="F71" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 2/3/4/8 containers of 1 vCPU, 2 GB (Fargate, Singapore).</t>
-        </is>
-      </c>
+          <t>BIR CAS registration support</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: books, system description, Permit to Use filing prepared with the broker. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="8" t="n"/>
       <c r="G71" s="8" t="n"/>
       <c r="H71" s="8" t="n"/>
       <c r="I71" s="8" t="n"/>
@@ -5139,26 +5177,24 @@
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>Managed PostgreSQL 16 (instance and storage)</t>
-        </is>
-      </c>
-      <c r="B72" s="16" t="n">
-        <v>85</v>
-      </c>
-      <c r="C72" s="16" t="n">
-        <v>320</v>
-      </c>
-      <c r="D72" s="16" t="n">
-        <v>640</v>
-      </c>
-      <c r="E72" s="16" t="n">
-        <v>1280</v>
-      </c>
-      <c r="F72" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: db.t4g.medium single-AZ / db.m7g.large Multi-AZ / m7g.xlarge Multi-AZ / m7g.2xlarge Multi-AZ (S20). Large and Enterprise: high availability.</t>
-        </is>
-      </c>
+          <t>BIR EIS enrolment and certification</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: enrolment, signing certificate, final field list, production endpoint and certification of the connector. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="n"/>
+      <c r="F72" s="8" t="n"/>
       <c r="G72" s="8" t="n"/>
       <c r="H72" s="8" t="n"/>
       <c r="I72" s="8" t="n"/>
@@ -5171,26 +5207,24 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>Object storage and backups (documents, snapshots)</t>
-        </is>
-      </c>
-      <c r="B73" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="C73" s="16" t="n">
-        <v>40</v>
-      </c>
-      <c r="D73" s="16" t="n">
-        <v>90</v>
-      </c>
-      <c r="E73" s="16" t="n">
-        <v>180</v>
-      </c>
-      <c r="F73" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: S3 and snapshot storage, growing with policies and uploads.</t>
-        </is>
-      </c>
+          <t>CTPL authentication and LTO interface certification</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: acceptance of the live requests by the accredited provider, COC series, LTO interface. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
       <c r="H73" s="8" t="n"/>
       <c r="I73" s="8" t="n"/>
@@ -5203,26 +5237,24 @@
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>Network (load balancer, CDN, data transfer)</t>
-        </is>
-      </c>
-      <c r="B74" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="C74" s="16" t="n">
-        <v>70</v>
-      </c>
-      <c r="D74" s="16" t="n">
-        <v>120</v>
-      </c>
-      <c r="E74" s="16" t="n">
-        <v>220</v>
-      </c>
-      <c r="F74" s="15" t="inlineStr">
-        <is>
-          <t>Estimate.</t>
-        </is>
-      </c>
+          <t>Insurer API onboarding, per insurer</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: endpoint, credentials, field mapping and live test with one insurer. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="n"/>
+      <c r="F74" s="8" t="n"/>
       <c r="G74" s="8" t="n"/>
       <c r="H74" s="8" t="n"/>
       <c r="I74" s="8" t="n"/>
@@ -5235,26 +5267,24 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>Security and monitoring (WAF, logs, alarms, secrets, keys)</t>
-        </is>
-      </c>
-      <c r="B75" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="C75" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="D75" s="16" t="n">
-        <v>110</v>
-      </c>
-      <c r="E75" s="16" t="n">
-        <v>200</v>
-      </c>
-      <c r="F75" s="15" t="inlineStr">
-        <is>
-          <t>Estimate.</t>
-        </is>
-      </c>
+          <t>Bank payment file certification, per bank</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: layout validated against the bank specification and a test file accepted. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="n"/>
+      <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="n"/>
       <c r="H75" s="8" t="n"/>
       <c r="I75" s="8" t="n"/>
@@ -5267,26 +5297,24 @@
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>Disaster recovery copy (cross-region backups)</t>
-        </is>
-      </c>
-      <c r="B76" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C76" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" s="16" t="n">
-        <v>400</v>
-      </c>
-      <c r="F76" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: Enterprise only; optional for others. Not part of Pre-Prod.</t>
-        </is>
-      </c>
+          <t>SMS or Viber gateway activation</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: sender name or short code, live credentials, templates and consent check tested. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="n"/>
+      <c r="F76" s="8" t="n"/>
       <c r="G76" s="8" t="n"/>
       <c r="H76" s="8" t="n"/>
       <c r="I76" s="8" t="n"/>
@@ -5297,32 +5325,39 @@
       <c r="N76" s="9" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="18" t="inlineStr">
-        <is>
-          <t>Production reference cost per month (USD)</t>
-        </is>
-      </c>
-      <c r="B77" s="21">
-        <f>SUM(B71:B76)</f>
-        <v/>
-      </c>
-      <c r="C77" s="21">
-        <f>SUM(C71:C76)</f>
-        <v/>
-      </c>
-      <c r="D77" s="21">
-        <f>SUM(D71:D76)</f>
-        <v/>
-      </c>
-      <c r="E77" s="21">
-        <f>SUM(E71:E76)</f>
-        <v/>
-      </c>
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>Screening list provider onboarding</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>man-days</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: provider contract data, API key, adapter test and first screening run. Optional service confirmed by management on 04 October 2026.</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="n"/>
+      <c r="F77" s="8" t="n"/>
+      <c r="G77" s="8" t="n"/>
+      <c r="H77" s="8" t="n"/>
+      <c r="I77" s="8" t="n"/>
+      <c r="J77" s="8" t="n"/>
+      <c r="K77" s="8" t="n"/>
+      <c r="L77" s="8" t="n"/>
+      <c r="M77" s="8" t="n"/>
+      <c r="N77" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure: non-production environment sizes and Pre-Prod use</t>
+          <t>Infrastructure: AWS reference cost per month of the Production environment (USD)</t>
         </is>
       </c>
       <c r="B79" s="7" t="n"/>
@@ -5342,26 +5377,34 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Driver</t>
+          <t>Component</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="8" t="n"/>
       <c r="G80" s="8" t="n"/>
       <c r="H80" s="8" t="n"/>
       <c r="I80" s="8" t="n"/>
@@ -5374,24 +5417,26 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>Non-production environment, small: cloud cost per month</t>
+          <t>Application containers (API, web, scheduler)</t>
         </is>
       </c>
       <c r="B81" s="16" t="n">
-        <v>150</v>
-      </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D81" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 1 container of 1 vCPU, 2 GB; PostgreSQL db.t4g.medium single-AZ, 50 GB; file store; backups 7 to 14 days. Dev in every tier; UAT of Small and Medium brokers.</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="n"/>
-      <c r="F81" s="8" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="C81" s="16" t="n">
+        <v>135</v>
+      </c>
+      <c r="D81" s="16" t="n">
+        <v>180</v>
+      </c>
+      <c r="E81" s="16" t="n">
+        <v>360</v>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 2/3/4/8 containers of 1 vCPU, 2 GB (Fargate, Singapore).</t>
+        </is>
+      </c>
       <c r="G81" s="8" t="n"/>
       <c r="H81" s="8" t="n"/>
       <c r="I81" s="8" t="n"/>
@@ -5404,24 +5449,26 @@
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
         <is>
-          <t>Non-production environment, medium: cloud cost per month</t>
+          <t>Managed PostgreSQL 16 (instance and storage)</t>
         </is>
       </c>
       <c r="B82" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>Estimate: 2 containers of 1 vCPU, 2 GB (the second for the UAT performance test); db.t4g.large single-AZ, 100 GB; file store; load balancer. SIT and UAT of Large and Enterprise brokers.</t>
-        </is>
-      </c>
-      <c r="E82" s="8" t="n"/>
-      <c r="F82" s="8" t="n"/>
+        <v>85</v>
+      </c>
+      <c r="C82" s="16" t="n">
+        <v>320</v>
+      </c>
+      <c r="D82" s="16" t="n">
+        <v>640</v>
+      </c>
+      <c r="E82" s="16" t="n">
+        <v>1280</v>
+      </c>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: db.t4g.medium single-AZ / db.m7g.large Multi-AZ / m7g.xlarge Multi-AZ / m7g.2xlarge Multi-AZ (S20). Large and Enterprise: high availability.</t>
+        </is>
+      </c>
       <c r="G82" s="8" t="n"/>
       <c r="H82" s="8" t="n"/>
       <c r="I82" s="8" t="n"/>
@@ -5434,24 +5481,26 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>Pre-Prod cloud cost relative to Production (without the DR copy)</t>
-        </is>
-      </c>
-      <c r="B83" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C83" s="10" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: Pre-Prod is restored from a production backup and runs at production topology and size, so the rehearsal measures real timings.</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="n"/>
-      <c r="F83" s="8" t="n"/>
+          <t>Object storage and backups (documents, snapshots)</t>
+        </is>
+      </c>
+      <c r="B83" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C83" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D83" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="E83" s="16" t="n">
+        <v>180</v>
+      </c>
+      <c r="F83" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: S3 and snapshot storage, growing with policies and uploads.</t>
+        </is>
+      </c>
       <c r="G83" s="8" t="n"/>
       <c r="H83" s="8" t="n"/>
       <c r="I83" s="8" t="n"/>
@@ -5464,24 +5513,26 @@
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>Pre-Prod months of use around go-live</t>
-        </is>
-      </c>
-      <c r="B84" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: created before the cutover rehearsal and removed after hypercare (1 to 2 months). Billed per month of use.</t>
-        </is>
-      </c>
-      <c r="E84" s="8" t="n"/>
-      <c r="F84" s="8" t="n"/>
+          <t>Network (load balancer, CDN, data transfer)</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="C84" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="D84" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="E84" s="16" t="n">
+        <v>220</v>
+      </c>
+      <c r="F84" s="15" t="inlineStr">
+        <is>
+          <t>Estimate.</t>
+        </is>
+      </c>
       <c r="G84" s="8" t="n"/>
       <c r="H84" s="8" t="n"/>
       <c r="I84" s="8" t="n"/>
@@ -5494,24 +5545,26 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Pre-Prod months of use per major release</t>
-        </is>
-      </c>
-      <c r="B85" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: created from a production backup for the release rehearsal and removed after the release.</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="n"/>
-      <c r="F85" s="8" t="n"/>
+          <t>Security and monitoring (WAF, logs, alarms, secrets, keys)</t>
+        </is>
+      </c>
+      <c r="B85" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="C85" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="D85" s="16" t="n">
+        <v>110</v>
+      </c>
+      <c r="E85" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="F85" s="15" t="inlineStr">
+        <is>
+          <t>Estimate.</t>
+        </is>
+      </c>
       <c r="G85" s="8" t="n"/>
       <c r="H85" s="8" t="n"/>
       <c r="I85" s="8" t="n"/>
@@ -5524,24 +5577,26 @@
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>Major releases per year (yearly hosting view only)</t>
-        </is>
-      </c>
-      <c r="B86" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>releases</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
-        <is>
-          <t>Assumption for budgeting. Major releases are announced at least 6 months ahead (Release Notes and Roadmap); the invoice follows the actual months of use.</t>
-        </is>
-      </c>
-      <c r="E86" s="8" t="n"/>
-      <c r="F86" s="8" t="n"/>
+          <t>Disaster recovery copy (cross-region backups)</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="F86" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: Enterprise only; optional for others. Not part of Pre-Prod.</t>
+        </is>
+      </c>
       <c r="G86" s="8" t="n"/>
       <c r="H86" s="8" t="n"/>
       <c r="I86" s="8" t="n"/>
@@ -5551,107 +5606,74 @@
       <c r="M86" s="8" t="n"/>
       <c r="N86" s="9" t="n"/>
     </row>
-    <row r="88">
-      <c r="A88" s="6" t="inlineStr">
-        <is>
-          <t>Infrastructure: environment set by tier, AWS reference cost per month (USD)</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="n"/>
-      <c r="C88" s="7" t="n"/>
-      <c r="D88" s="7" t="n"/>
-      <c r="E88" s="7" t="n"/>
-      <c r="F88" s="7" t="n"/>
-      <c r="G88" s="7" t="n"/>
-      <c r="H88" s="7" t="n"/>
-      <c r="I88" s="7" t="n"/>
-      <c r="J88" s="7" t="n"/>
-      <c r="K88" s="7" t="n"/>
-      <c r="L88" s="7" t="n"/>
-      <c r="M88" s="7" t="n"/>
-      <c r="N88" s="7" t="n"/>
-    </row>
-    <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Dev</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>SIT</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="F89" s="3" t="inlineStr">
-        <is>
-          <t>Standing environments</t>
-        </is>
-      </c>
-      <c r="G89" s="3" t="inlineStr">
-        <is>
-          <t>Pre-Prod per month of use</t>
-        </is>
-      </c>
-      <c r="H89" s="3" t="inlineStr">
-        <is>
-          <t>Environment set and basis</t>
-        </is>
-      </c>
-      <c r="I89" s="8" t="n"/>
-      <c r="J89" s="8" t="n"/>
-      <c r="K89" s="8" t="n"/>
-      <c r="L89" s="8" t="n"/>
-      <c r="M89" s="8" t="n"/>
-      <c r="N89" s="9" t="n"/>
+    <row r="87">
+      <c r="A87" s="18" t="inlineStr">
+        <is>
+          <t>Production reference cost per month (USD)</t>
+        </is>
+      </c>
+      <c r="B87" s="21">
+        <f>SUM(B81:B86)</f>
+        <v/>
+      </c>
+      <c r="C87" s="21">
+        <f>SUM(C81:C86)</f>
+        <v/>
+      </c>
+      <c r="D87" s="21">
+        <f>SUM(D81:D86)</f>
+        <v/>
+      </c>
+      <c r="E87" s="21">
+        <f>SUM(E81:E86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>Infrastructure: non-production environment sizes and Pre-Prod use</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="n"/>
+      <c r="C89" s="7" t="n"/>
+      <c r="D89" s="7" t="n"/>
+      <c r="E89" s="7" t="n"/>
+      <c r="F89" s="7" t="n"/>
+      <c r="G89" s="7" t="n"/>
+      <c r="H89" s="7" t="n"/>
+      <c r="I89" s="7" t="n"/>
+      <c r="J89" s="7" t="n"/>
+      <c r="K89" s="7" t="n"/>
+      <c r="L89" s="7" t="n"/>
+      <c r="M89" s="7" t="n"/>
+      <c r="N89" s="7" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="18">
-        <f>A28</f>
-        <v/>
-      </c>
-      <c r="B90" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C90" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D90" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="E90" s="20">
-        <f>B77</f>
-        <v/>
-      </c>
-      <c r="F90" s="24">
-        <f>SUM(B90:E90)</f>
-        <v/>
-      </c>
-      <c r="G90" s="21">
-        <f>SUM(B71:B75)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H90" s="5" t="inlineStr">
-        <is>
-          <t>Dev, UAT, Production, temporary Pre-Prod. Integration and SIT in Dev, then promoted to UAT for testing.</t>
-        </is>
-      </c>
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="n"/>
+      <c r="F90" s="8" t="n"/>
+      <c r="G90" s="8" t="n"/>
+      <c r="H90" s="8" t="n"/>
       <c r="I90" s="8" t="n"/>
       <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="n"/>
@@ -5660,38 +5682,28 @@
       <c r="N90" s="9" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="18">
-        <f>A29</f>
-        <v/>
-      </c>
-      <c r="B91" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C91" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D91" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="E91" s="20">
-        <f>C77</f>
-        <v/>
-      </c>
-      <c r="F91" s="24">
-        <f>SUM(B91:E91)</f>
-        <v/>
-      </c>
-      <c r="G91" s="21">
-        <f>SUM(C71:C75)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H91" s="5" t="inlineStr">
-        <is>
-          <t>Dev, UAT, Production, temporary Pre-Prod. As Small.</t>
-        </is>
-      </c>
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>Non-production environment, small: cloud cost per month</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 1 container of 1 vCPU, 2 GB; PostgreSQL db.t4g.medium single-AZ, 50 GB; file store; backups 7 to 14 days. Dev in every tier; UAT of Small and Medium brokers.</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="n"/>
+      <c r="F91" s="8" t="n"/>
+      <c r="G91" s="8" t="n"/>
+      <c r="H91" s="8" t="n"/>
       <c r="I91" s="8" t="n"/>
       <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="n"/>
@@ -5700,39 +5712,28 @@
       <c r="N91" s="9" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="18">
-        <f>A30</f>
-        <v/>
-      </c>
-      <c r="B92" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C92" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="D92" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="E92" s="20">
-        <f>D77</f>
-        <v/>
-      </c>
-      <c r="F92" s="24">
-        <f>SUM(B92:E92)</f>
-        <v/>
-      </c>
-      <c r="G92" s="21">
-        <f>SUM(D71:D75)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H92" s="5" t="inlineStr">
-        <is>
-          <t>Dev, SIT, UAT, Production with high availability, temporary Pre-Prod. SIT and UAT are separate.</t>
-        </is>
-      </c>
+      <c r="A92" s="10" t="inlineStr">
+        <is>
+          <t>Non-production environment, medium: cloud cost per month</t>
+        </is>
+      </c>
+      <c r="B92" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
+        <is>
+          <t>Estimate: 2 containers of 1 vCPU, 2 GB (the second for the UAT performance test); db.t4g.large single-AZ, 100 GB; file store; load balancer. SIT and UAT of Large and Enterprise brokers.</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="n"/>
+      <c r="F92" s="8" t="n"/>
+      <c r="G92" s="8" t="n"/>
+      <c r="H92" s="8" t="n"/>
       <c r="I92" s="8" t="n"/>
       <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="n"/>
@@ -5741,39 +5742,28 @@
       <c r="N92" s="9" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="18">
-        <f>A31</f>
-        <v/>
-      </c>
-      <c r="B93" s="20">
-        <f>NP_Small_USD</f>
-        <v/>
-      </c>
-      <c r="C93" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="D93" s="20">
-        <f>NP_Med_USD</f>
-        <v/>
-      </c>
-      <c r="E93" s="20">
-        <f>E77</f>
-        <v/>
-      </c>
-      <c r="F93" s="24">
-        <f>SUM(B93:E93)</f>
-        <v/>
-      </c>
-      <c r="G93" s="21">
-        <f>SUM(E71:E75)*PreProd_Factor</f>
-        <v/>
-      </c>
-      <c r="H93" s="5" t="inlineStr">
-        <is>
-          <t>As Large, with the cross-region DR copy in Production.</t>
-        </is>
-      </c>
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Pre-Prod cloud cost relative to Production (without the DR copy)</t>
+        </is>
+      </c>
+      <c r="B93" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: Pre-Prod is restored from a production backup and runs at production topology and size, so the rehearsal measures real timings.</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="n"/>
+      <c r="F93" s="8" t="n"/>
+      <c r="G93" s="8" t="n"/>
+      <c r="H93" s="8" t="n"/>
       <c r="I93" s="8" t="n"/>
       <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="n"/>
@@ -5784,17 +5774,24 @@
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>Azure cost relative to AWS</t>
-        </is>
-      </c>
-      <c r="B94" s="11" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="F94" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: comparable list prices in Southeast Asia (D4s v5 Linux about USD 158 a month, S21); +5% for managed PostgreSQL and WAF differences.</t>
-        </is>
-      </c>
+          <t>Pre-Prod months of use around go-live</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: created before the cutover rehearsal and removed after hypercare (1 to 2 months). Billed per month of use.</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="n"/>
+      <c r="F94" s="8" t="n"/>
       <c r="G94" s="8" t="n"/>
       <c r="H94" s="8" t="n"/>
       <c r="I94" s="8" t="n"/>
@@ -5807,17 +5804,24 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>Local partner cloud cost relative to AWS</t>
-        </is>
-      </c>
-      <c r="B95" s="11" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F95" s="15" t="inlineStr">
-        <is>
-          <t>Assumption: Philippine data-centre or partner cloud priced in PHP; lower compute and bandwidth, database run as managed VM. Confirm with a partner quotation.</t>
-        </is>
-      </c>
+          <t>Pre-Prod months of use per major release</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: created from a production backup for the release rehearsal and removed after the release.</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="n"/>
+      <c r="F95" s="8" t="n"/>
       <c r="G95" s="8" t="n"/>
       <c r="H95" s="8" t="n"/>
       <c r="I95" s="8" t="n"/>
@@ -5827,90 +5831,97 @@
       <c r="M95" s="8" t="n"/>
       <c r="N95" s="9" t="n"/>
     </row>
-    <row r="97">
-      <c r="A97" s="6" t="inlineStr">
-        <is>
-          <t>Sample quote scenarios (used by Sample Quotes)</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="n"/>
-      <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
-      <c r="E97" s="7" t="n"/>
-      <c r="F97" s="7" t="n"/>
-      <c r="G97" s="7" t="n"/>
-      <c r="H97" s="7" t="n"/>
-      <c r="I97" s="7" t="n"/>
-      <c r="J97" s="7" t="n"/>
-      <c r="K97" s="7" t="n"/>
-      <c r="L97" s="7" t="n"/>
-      <c r="M97" s="7" t="n"/>
-      <c r="N97" s="7" t="n"/>
+    <row r="96">
+      <c r="A96" s="10" t="inlineStr">
+        <is>
+          <t>Major releases per year (yearly hosting view only)</t>
+        </is>
+      </c>
+      <c r="B96" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>releases</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>Assumption for budgeting. Major releases are announced at least 6 months ahead (Release Notes and Roadmap); the invoice follows the actual months of use.</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="n"/>
+      <c r="F96" s="8" t="n"/>
+      <c r="G96" s="8" t="n"/>
+      <c r="H96" s="8" t="n"/>
+      <c r="I96" s="8" t="n"/>
+      <c r="J96" s="8" t="n"/>
+      <c r="K96" s="8" t="n"/>
+      <c r="L96" s="8" t="n"/>
+      <c r="M96" s="8" t="n"/>
+      <c r="N96" s="9" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="3" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="C98" s="3" t="inlineStr">
-        <is>
-          <t>Example 2</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>Example 3</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr"/>
-      <c r="F98" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G98" s="8" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
-      <c r="J98" s="8" t="n"/>
-      <c r="K98" s="8" t="n"/>
-      <c r="L98" s="8" t="n"/>
-      <c r="M98" s="8" t="n"/>
-      <c r="N98" s="9" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="10" t="inlineStr">
-        <is>
-          <t>Broker profile</t>
-        </is>
-      </c>
-      <c r="B99" s="12" t="inlineStr">
-        <is>
-          <t>Small broker</t>
-        </is>
-      </c>
-      <c r="C99" s="12" t="inlineStr">
-        <is>
-          <t>Medium broker</t>
-        </is>
-      </c>
-      <c r="D99" s="12" t="inlineStr">
-        <is>
-          <t>Large broker</t>
-        </is>
-      </c>
-      <c r="F99" s="10" t="inlineStr">
-        <is>
-          <t>Label only.</t>
-        </is>
-      </c>
-      <c r="G99" s="8" t="n"/>
-      <c r="H99" s="8" t="n"/>
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Infrastructure: environment set by tier, AWS reference cost per month (USD)</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="n"/>
+      <c r="C98" s="7" t="n"/>
+      <c r="D98" s="7" t="n"/>
+      <c r="E98" s="7" t="n"/>
+      <c r="F98" s="7" t="n"/>
+      <c r="G98" s="7" t="n"/>
+      <c r="H98" s="7" t="n"/>
+      <c r="I98" s="7" t="n"/>
+      <c r="J98" s="7" t="n"/>
+      <c r="K98" s="7" t="n"/>
+      <c r="L98" s="7" t="n"/>
+      <c r="M98" s="7" t="n"/>
+      <c r="N98" s="7" t="n"/>
+    </row>
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>SIT</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Standing environments</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Prod per month of use</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Environment set and basis</t>
+        </is>
+      </c>
       <c r="I99" s="8" t="n"/>
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
@@ -5919,27 +5930,38 @@
       <c r="N99" s="9" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="10" t="inlineStr">
-        <is>
-          <t>Named users</t>
-        </is>
-      </c>
-      <c r="B100" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C100" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="D100" s="14" t="n">
-        <v>180</v>
-      </c>
-      <c r="F100" s="10" t="inlineStr">
-        <is>
-          <t>Tier follows from the user count.</t>
-        </is>
-      </c>
-      <c r="G100" s="8" t="n"/>
-      <c r="H100" s="8" t="n"/>
+      <c r="A100" s="18">
+        <f>A28</f>
+        <v/>
+      </c>
+      <c r="B100" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C100" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="E100" s="20">
+        <f>B87</f>
+        <v/>
+      </c>
+      <c r="F100" s="24">
+        <f>SUM(B100:E100)</f>
+        <v/>
+      </c>
+      <c r="G100" s="21">
+        <f>SUM(B81:B85)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>Dev, UAT, Production, temporary Pre-Prod. Integration and SIT in Dev, then promoted to UAT for testing.</t>
+        </is>
+      </c>
       <c r="I100" s="8" t="n"/>
       <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="n"/>
@@ -5948,27 +5970,38 @@
       <c r="N100" s="9" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="10" t="inlineStr">
-        <is>
-          <t>Lines of business</t>
-        </is>
-      </c>
-      <c r="B101" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C101" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="D101" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="F101" s="10" t="inlineStr">
-        <is>
-          <t>Motor, fire, marine, casualty, engineering, bonds and so on.</t>
-        </is>
-      </c>
-      <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="n"/>
+      <c r="A101" s="18">
+        <f>A29</f>
+        <v/>
+      </c>
+      <c r="B101" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C101" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="E101" s="20">
+        <f>C87</f>
+        <v/>
+      </c>
+      <c r="F101" s="24">
+        <f>SUM(B101:E101)</f>
+        <v/>
+      </c>
+      <c r="G101" s="21">
+        <f>SUM(C81:C85)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>Dev, UAT, Production, temporary Pre-Prod. As Small.</t>
+        </is>
+      </c>
       <c r="I101" s="8" t="n"/>
       <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="n"/>
@@ -5977,33 +6010,39 @@
       <c r="N101" s="9" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="10" t="inlineStr">
-        <is>
-          <t>Infrastructure provider (AWS, Azure, Local partner, Customer)</t>
-        </is>
-      </c>
-      <c r="B102" s="12" t="inlineStr">
-        <is>
-          <t>AWS</t>
-        </is>
-      </c>
-      <c r="C102" s="12" t="inlineStr">
-        <is>
-          <t>Azure</t>
-        </is>
-      </c>
-      <c r="D102" s="12" t="inlineStr">
-        <is>
-          <t>Local partner</t>
-        </is>
-      </c>
-      <c r="F102" s="10" t="inlineStr">
-        <is>
-          <t>"Customer" means the broker hosts itself: no infrastructure fee.</t>
-        </is>
-      </c>
-      <c r="G102" s="8" t="n"/>
-      <c r="H102" s="8" t="n"/>
+      <c r="A102" s="18">
+        <f>A30</f>
+        <v/>
+      </c>
+      <c r="B102" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C102" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="D102" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="E102" s="20">
+        <f>D87</f>
+        <v/>
+      </c>
+      <c r="F102" s="24">
+        <f>SUM(B102:E102)</f>
+        <v/>
+      </c>
+      <c r="G102" s="21">
+        <f>SUM(D81:D85)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>Dev, SIT, UAT, Production with high availability, temporary Pre-Prod. SIT and UAT are separate.</t>
+        </is>
+      </c>
       <c r="I102" s="8" t="n"/>
       <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="n"/>
@@ -6012,33 +6051,39 @@
       <c r="N102" s="9" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="inlineStr">
-        <is>
-          <t>24x7 Severity 1 support (Yes/No)</t>
-        </is>
-      </c>
-      <c r="B103" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C103" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D103" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F103" s="10" t="inlineStr">
-        <is>
-          <t>Optional.</t>
-        </is>
-      </c>
-      <c r="G103" s="8" t="n"/>
-      <c r="H103" s="8" t="n"/>
+      <c r="A103" s="18">
+        <f>A31</f>
+        <v/>
+      </c>
+      <c r="B103" s="20">
+        <f>NP_Small_USD</f>
+        <v/>
+      </c>
+      <c r="C103" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="D103" s="20">
+        <f>NP_Med_USD</f>
+        <v/>
+      </c>
+      <c r="E103" s="20">
+        <f>E87</f>
+        <v/>
+      </c>
+      <c r="F103" s="24">
+        <f>SUM(B103:E103)</f>
+        <v/>
+      </c>
+      <c r="G103" s="21">
+        <f>SUM(E81:E85)*PreProd_Factor</f>
+        <v/>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>As Large, with the cross-region DR copy in Production.</t>
+        </is>
+      </c>
       <c r="I103" s="8" t="n"/>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
@@ -6049,21 +6094,15 @@
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>Extra training days</t>
-        </is>
-      </c>
-      <c r="B104" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C104" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D104" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F104" s="10" t="inlineStr">
-        <is>
-          <t>Beyond the days included for the tier.</t>
+          <t>Azure cost relative to AWS</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: comparable list prices in Southeast Asia (D4s v5 Linux about USD 158 a month, S21); +5% for managed PostgreSQL and WAF differences.</t>
         </is>
       </c>
       <c r="G104" s="8" t="n"/>
@@ -6078,21 +6117,15 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Extra legacy data sources to migrate</t>
-        </is>
-      </c>
-      <c r="B105" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D105" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F105" s="10" t="inlineStr">
-        <is>
-          <t>Beyond the standard templates.</t>
+          <t>Local partner cloud cost relative to AWS</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F105" s="15" t="inlineStr">
+        <is>
+          <t>Assumption: Philippine data-centre or partner cloud priced in PHP; lower compute and bandwidth, database run as managed VM. Confirm with a partner quotation.</t>
         </is>
       </c>
       <c r="G105" s="8" t="n"/>
@@ -6104,117 +6137,404 @@
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="9" t="n"/>
     </row>
-    <row r="106">
-      <c r="A106" s="10" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>Sample quote scenarios (used by Sample Quotes)</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="n"/>
+      <c r="C107" s="7" t="n"/>
+      <c r="D107" s="7" t="n"/>
+      <c r="E107" s="7" t="n"/>
+      <c r="F107" s="7" t="n"/>
+      <c r="G107" s="7" t="n"/>
+      <c r="H107" s="7" t="n"/>
+      <c r="I107" s="7" t="n"/>
+      <c r="J107" s="7" t="n"/>
+      <c r="K107" s="7" t="n"/>
+      <c r="L107" s="7" t="n"/>
+      <c r="M107" s="7" t="n"/>
+      <c r="N107" s="7" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Example 1</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Example 2</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Example 3</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr"/>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="n"/>
+      <c r="H108" s="8" t="n"/>
+      <c r="I108" s="8" t="n"/>
+      <c r="J108" s="8" t="n"/>
+      <c r="K108" s="8" t="n"/>
+      <c r="L108" s="8" t="n"/>
+      <c r="M108" s="8" t="n"/>
+      <c r="N108" s="9" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>Broker profile</t>
+        </is>
+      </c>
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>Small broker</t>
+        </is>
+      </c>
+      <c r="C109" s="12" t="inlineStr">
+        <is>
+          <t>Medium broker</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="inlineStr">
+        <is>
+          <t>Large broker</t>
+        </is>
+      </c>
+      <c r="F109" s="10" t="inlineStr">
+        <is>
+          <t>Label only.</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="n"/>
+      <c r="H109" s="8" t="n"/>
+      <c r="I109" s="8" t="n"/>
+      <c r="J109" s="8" t="n"/>
+      <c r="K109" s="8" t="n"/>
+      <c r="L109" s="8" t="n"/>
+      <c r="M109" s="8" t="n"/>
+      <c r="N109" s="9" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
+          <t>Named users</t>
+        </is>
+      </c>
+      <c r="B110" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="C110" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D110" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="F110" s="10" t="inlineStr">
+        <is>
+          <t>Tier follows from the user count.</t>
+        </is>
+      </c>
+      <c r="G110" s="8" t="n"/>
+      <c r="H110" s="8" t="n"/>
+      <c r="I110" s="8" t="n"/>
+      <c r="J110" s="8" t="n"/>
+      <c r="K110" s="8" t="n"/>
+      <c r="L110" s="8" t="n"/>
+      <c r="M110" s="8" t="n"/>
+      <c r="N110" s="9" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Lines of business</t>
+        </is>
+      </c>
+      <c r="B111" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C111" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D111" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>Motor, fire, marine, casualty, engineering, bonds and so on.</t>
+        </is>
+      </c>
+      <c r="G111" s="8" t="n"/>
+      <c r="H111" s="8" t="n"/>
+      <c r="I111" s="8" t="n"/>
+      <c r="J111" s="8" t="n"/>
+      <c r="K111" s="8" t="n"/>
+      <c r="L111" s="8" t="n"/>
+      <c r="M111" s="8" t="n"/>
+      <c r="N111" s="9" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>Infrastructure provider (AWS, Azure, Local partner, Customer)</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="inlineStr">
+        <is>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="D112" s="12" t="inlineStr">
+        <is>
+          <t>Local partner</t>
+        </is>
+      </c>
+      <c r="F112" s="10" t="inlineStr">
+        <is>
+          <t>"Customer" means the broker hosts itself: no infrastructure fee.</t>
+        </is>
+      </c>
+      <c r="G112" s="8" t="n"/>
+      <c r="H112" s="8" t="n"/>
+      <c r="I112" s="8" t="n"/>
+      <c r="J112" s="8" t="n"/>
+      <c r="K112" s="8" t="n"/>
+      <c r="L112" s="8" t="n"/>
+      <c r="M112" s="8" t="n"/>
+      <c r="N112" s="9" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>24x7 Severity 1 support (Yes/No)</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F113" s="10" t="inlineStr">
+        <is>
+          <t>Optional.</t>
+        </is>
+      </c>
+      <c r="G113" s="8" t="n"/>
+      <c r="H113" s="8" t="n"/>
+      <c r="I113" s="8" t="n"/>
+      <c r="J113" s="8" t="n"/>
+      <c r="K113" s="8" t="n"/>
+      <c r="L113" s="8" t="n"/>
+      <c r="M113" s="8" t="n"/>
+      <c r="N113" s="9" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Extra training days</t>
+        </is>
+      </c>
+      <c r="B114" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D114" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F114" s="10" t="inlineStr">
+        <is>
+          <t>Beyond the days included for the tier.</t>
+        </is>
+      </c>
+      <c r="G114" s="8" t="n"/>
+      <c r="H114" s="8" t="n"/>
+      <c r="I114" s="8" t="n"/>
+      <c r="J114" s="8" t="n"/>
+      <c r="K114" s="8" t="n"/>
+      <c r="L114" s="8" t="n"/>
+      <c r="M114" s="8" t="n"/>
+      <c r="N114" s="9" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Extra legacy data sources to migrate</t>
+        </is>
+      </c>
+      <c r="B115" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C115" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
+          <t>Beyond the standard templates.</t>
+        </is>
+      </c>
+      <c r="G115" s="8" t="n"/>
+      <c r="H115" s="8" t="n"/>
+      <c r="I115" s="8" t="n"/>
+      <c r="J115" s="8" t="n"/>
+      <c r="K115" s="8" t="n"/>
+      <c r="L115" s="8" t="n"/>
+      <c r="M115" s="8" t="n"/>
+      <c r="N115" s="9" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
         <is>
           <t>Additional standard integrations</t>
         </is>
       </c>
-      <c r="B106" s="14" t="n">
+      <c r="B116" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C106" s="14" t="n">
+      <c r="C116" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D106" s="14" t="n">
+      <c r="D116" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F106" s="10" t="inlineStr">
+      <c r="F116" s="10" t="inlineStr">
         <is>
           <t>One-time.</t>
         </is>
       </c>
-      <c r="G106" s="8" t="n"/>
-      <c r="H106" s="8" t="n"/>
-      <c r="I106" s="8" t="n"/>
-      <c r="J106" s="8" t="n"/>
-      <c r="K106" s="8" t="n"/>
-      <c r="L106" s="8" t="n"/>
-      <c r="M106" s="8" t="n"/>
-      <c r="N106" s="9" t="n"/>
+      <c r="G116" s="8" t="n"/>
+      <c r="H116" s="8" t="n"/>
+      <c r="I116" s="8" t="n"/>
+      <c r="J116" s="8" t="n"/>
+      <c r="K116" s="8" t="n"/>
+      <c r="L116" s="8" t="n"/>
+      <c r="M116" s="8" t="n"/>
+      <c r="N116" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="74">
-    <mergeCell ref="E36:N36"/>
+  <mergeCells count="84">
     <mergeCell ref="D59:N59"/>
-    <mergeCell ref="D50:N50"/>
-    <mergeCell ref="F104:N104"/>
+    <mergeCell ref="F86:N86"/>
+    <mergeCell ref="F80:N80"/>
     <mergeCell ref="D60:N60"/>
-    <mergeCell ref="F76:N76"/>
-    <mergeCell ref="F95:N95"/>
-    <mergeCell ref="D19:N19"/>
-    <mergeCell ref="D63:N63"/>
-    <mergeCell ref="F94:N94"/>
-    <mergeCell ref="D10:N10"/>
-    <mergeCell ref="F101:N101"/>
-    <mergeCell ref="F70:N70"/>
-    <mergeCell ref="D81:N81"/>
-    <mergeCell ref="D46:N46"/>
-    <mergeCell ref="D84:N84"/>
-    <mergeCell ref="F75:N75"/>
-    <mergeCell ref="F106:N106"/>
-    <mergeCell ref="D80:N80"/>
-    <mergeCell ref="E41:N41"/>
-    <mergeCell ref="D65:N65"/>
     <mergeCell ref="D45:N45"/>
-    <mergeCell ref="F100:N100"/>
-    <mergeCell ref="F72:N72"/>
-    <mergeCell ref="E37:N37"/>
     <mergeCell ref="D6:N6"/>
-    <mergeCell ref="D52:N52"/>
-    <mergeCell ref="H92:N92"/>
-    <mergeCell ref="D86:N86"/>
-    <mergeCell ref="D11:N11"/>
-    <mergeCell ref="D49:N49"/>
-    <mergeCell ref="D57:N57"/>
-    <mergeCell ref="H91:N91"/>
-    <mergeCell ref="F102:N102"/>
-    <mergeCell ref="F71:N71"/>
-    <mergeCell ref="D13:N13"/>
+    <mergeCell ref="F81:N81"/>
+    <mergeCell ref="D95:N95"/>
     <mergeCell ref="F105:N105"/>
+    <mergeCell ref="D70:N70"/>
     <mergeCell ref="E42:N42"/>
     <mergeCell ref="D48:N48"/>
+    <mergeCell ref="D7:N7"/>
+    <mergeCell ref="D72:N72"/>
+    <mergeCell ref="D62:N62"/>
+    <mergeCell ref="D56:N56"/>
+    <mergeCell ref="D71:N71"/>
+    <mergeCell ref="D58:N58"/>
+    <mergeCell ref="D64:N64"/>
+    <mergeCell ref="D73:N73"/>
+    <mergeCell ref="D51:N51"/>
+    <mergeCell ref="F83:N83"/>
+    <mergeCell ref="D50:N50"/>
+    <mergeCell ref="F85:N85"/>
+    <mergeCell ref="D19:N19"/>
+    <mergeCell ref="D90:N90"/>
+    <mergeCell ref="F109:N109"/>
+    <mergeCell ref="E41:N41"/>
+    <mergeCell ref="D77:N77"/>
+    <mergeCell ref="D11:N11"/>
+    <mergeCell ref="F111:N111"/>
+    <mergeCell ref="D13:N13"/>
+    <mergeCell ref="D61:N61"/>
+    <mergeCell ref="D75:N75"/>
+    <mergeCell ref="D53:N53"/>
+    <mergeCell ref="D47:N47"/>
+    <mergeCell ref="E35:N35"/>
+    <mergeCell ref="A32:N32"/>
+    <mergeCell ref="D9:N9"/>
+    <mergeCell ref="D15:N15"/>
+    <mergeCell ref="H100:N100"/>
+    <mergeCell ref="E36:N36"/>
+    <mergeCell ref="F114:N114"/>
+    <mergeCell ref="D63:N63"/>
+    <mergeCell ref="D10:N10"/>
+    <mergeCell ref="F110:N110"/>
+    <mergeCell ref="D65:N65"/>
+    <mergeCell ref="E37:N37"/>
+    <mergeCell ref="D52:N52"/>
+    <mergeCell ref="F115:N115"/>
+    <mergeCell ref="D49:N49"/>
+    <mergeCell ref="D76:N76"/>
+    <mergeCell ref="H103:N103"/>
     <mergeCell ref="D17:N17"/>
-    <mergeCell ref="D61:N61"/>
-    <mergeCell ref="D53:N53"/>
+    <mergeCell ref="D91:N91"/>
     <mergeCell ref="D66:N66"/>
-    <mergeCell ref="H93:N93"/>
+    <mergeCell ref="D93:N93"/>
+    <mergeCell ref="D12:N12"/>
+    <mergeCell ref="F112:N112"/>
+    <mergeCell ref="D92:N92"/>
+    <mergeCell ref="D67:N67"/>
+    <mergeCell ref="D5:N5"/>
+    <mergeCell ref="D14:N14"/>
+    <mergeCell ref="D94:N94"/>
+    <mergeCell ref="H99:N99"/>
+    <mergeCell ref="D69:N69"/>
+    <mergeCell ref="F104:N104"/>
+    <mergeCell ref="F113:N113"/>
+    <mergeCell ref="H101:N101"/>
+    <mergeCell ref="D46:N46"/>
+    <mergeCell ref="D96:N96"/>
+    <mergeCell ref="D57:N57"/>
+    <mergeCell ref="H102:N102"/>
+    <mergeCell ref="F82:N82"/>
     <mergeCell ref="E39:N39"/>
     <mergeCell ref="D16:N16"/>
-    <mergeCell ref="D47:N47"/>
-    <mergeCell ref="F98:N98"/>
-    <mergeCell ref="D7:N7"/>
-    <mergeCell ref="E35:N35"/>
     <mergeCell ref="E38:N38"/>
-    <mergeCell ref="D62:N62"/>
-    <mergeCell ref="A32:N32"/>
-    <mergeCell ref="F73:N73"/>
     <mergeCell ref="D18:N18"/>
-    <mergeCell ref="D56:N56"/>
-    <mergeCell ref="H89:N89"/>
-    <mergeCell ref="D9:N9"/>
-    <mergeCell ref="D12:N12"/>
-    <mergeCell ref="D58:N58"/>
+    <mergeCell ref="F116:N116"/>
     <mergeCell ref="D8:N8"/>
-    <mergeCell ref="D83:N83"/>
-    <mergeCell ref="F103:N103"/>
-    <mergeCell ref="D64:N64"/>
-    <mergeCell ref="D15:N15"/>
-    <mergeCell ref="D82:N82"/>
-    <mergeCell ref="F99:N99"/>
-    <mergeCell ref="D67:N67"/>
-    <mergeCell ref="D5:N5"/>
-    <mergeCell ref="D51:N51"/>
-    <mergeCell ref="F74:N74"/>
-    <mergeCell ref="D14:N14"/>
-    <mergeCell ref="D85:N85"/>
-    <mergeCell ref="H90:N90"/>
+    <mergeCell ref="D74:N74"/>
+    <mergeCell ref="F108:N108"/>
+    <mergeCell ref="D68:N68"/>
+    <mergeCell ref="F84:N84"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B102:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B112:D112" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"AWS,Azure,Local partner,Customer"</formula1>
     </dataValidation>
-    <dataValidation sqref="B103:D103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B113:D113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10435,19 +10755,19 @@
         </is>
       </c>
       <c r="D5" s="27">
-        <f>ROUND(Inputs!B90*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B100*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E5" s="27">
-        <f>ROUND(Inputs!C90*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C100*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F5" s="27">
-        <f>ROUND(Inputs!D90*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D100*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G5" s="27">
-        <f>ROUND(Inputs!E90*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E100*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H5" s="24">
@@ -10455,7 +10775,7 @@
         <v/>
       </c>
       <c r="I5" s="24">
-        <f>ROUND(Inputs!G90*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G100*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J5" s="20">
@@ -10492,19 +10812,19 @@
         </is>
       </c>
       <c r="D6" s="27">
-        <f>ROUND(Inputs!B91*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B101*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E6" s="27">
-        <f>ROUND(Inputs!C91*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C101*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F6" s="27">
-        <f>ROUND(Inputs!D91*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D101*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G6" s="27">
-        <f>ROUND(Inputs!E91*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E101*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H6" s="24">
@@ -10512,7 +10832,7 @@
         <v/>
       </c>
       <c r="I6" s="24">
-        <f>ROUND(Inputs!G91*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G101*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J6" s="20">
@@ -10545,19 +10865,19 @@
         </is>
       </c>
       <c r="D7" s="27">
-        <f>ROUND(Inputs!B92*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B102*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E7" s="27">
-        <f>ROUND(Inputs!C92*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C102*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F7" s="27">
-        <f>ROUND(Inputs!D92*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D102*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G7" s="27">
-        <f>ROUND(Inputs!E92*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E102*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H7" s="24">
@@ -10565,7 +10885,7 @@
         <v/>
       </c>
       <c r="I7" s="24">
-        <f>ROUND(Inputs!G92*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G102*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J7" s="20">
@@ -10598,19 +10918,19 @@
         </is>
       </c>
       <c r="D8" s="27">
-        <f>ROUND(Inputs!B93*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B103*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E8" s="27">
-        <f>ROUND(Inputs!C93*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C103*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F8" s="27">
-        <f>ROUND(Inputs!D93*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D103*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G8" s="27">
-        <f>ROUND(Inputs!E93*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E103*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H8" s="24">
@@ -10618,7 +10938,7 @@
         <v/>
       </c>
       <c r="I8" s="24">
-        <f>ROUND(Inputs!G93*1*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G103*1*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J8" s="20">
@@ -10651,19 +10971,19 @@
         </is>
       </c>
       <c r="D9" s="27">
-        <f>ROUND(Inputs!B90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B100*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E9" s="27">
-        <f>ROUND(Inputs!C90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C100*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F9" s="27">
-        <f>ROUND(Inputs!D90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D100*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G9" s="27">
-        <f>ROUND(Inputs!E90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E100*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H9" s="24">
@@ -10671,7 +10991,7 @@
         <v/>
       </c>
       <c r="I9" s="24">
-        <f>ROUND(Inputs!G90*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G100*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J9" s="20">
@@ -10708,19 +11028,19 @@
         </is>
       </c>
       <c r="D10" s="27">
-        <f>ROUND(Inputs!B91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B101*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>ROUND(Inputs!C91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C101*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>ROUND(Inputs!D91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D101*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>ROUND(Inputs!E91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E101*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H10" s="24">
@@ -10728,7 +11048,7 @@
         <v/>
       </c>
       <c r="I10" s="24">
-        <f>ROUND(Inputs!G91*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G101*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J10" s="20">
@@ -10761,19 +11081,19 @@
         </is>
       </c>
       <c r="D11" s="27">
-        <f>ROUND(Inputs!B92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B102*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E11" s="27">
-        <f>ROUND(Inputs!C92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C102*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F11" s="27">
-        <f>ROUND(Inputs!D92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D102*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G11" s="27">
-        <f>ROUND(Inputs!E92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E102*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H11" s="24">
@@ -10781,7 +11101,7 @@
         <v/>
       </c>
       <c r="I11" s="24">
-        <f>ROUND(Inputs!G92*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G102*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J11" s="20">
@@ -10814,19 +11134,19 @@
         </is>
       </c>
       <c r="D12" s="27">
-        <f>ROUND(Inputs!B93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B103*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E12" s="27">
-        <f>ROUND(Inputs!C93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C103*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F12" s="27">
-        <f>ROUND(Inputs!D93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D103*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G12" s="27">
-        <f>ROUND(Inputs!E93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E103*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H12" s="24">
@@ -10834,7 +11154,7 @@
         <v/>
       </c>
       <c r="I12" s="24">
-        <f>ROUND(Inputs!G93*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G103*Azure_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J12" s="20">
@@ -10867,19 +11187,19 @@
         </is>
       </c>
       <c r="D13" s="27">
-        <f>ROUND(Inputs!B90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B100*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E13" s="27">
-        <f>ROUND(Inputs!C90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C100*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F13" s="27">
-        <f>ROUND(Inputs!D90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D100*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G13" s="27">
-        <f>ROUND(Inputs!E90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E100*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H13" s="24">
@@ -10887,7 +11207,7 @@
         <v/>
       </c>
       <c r="I13" s="24">
-        <f>ROUND(Inputs!G90*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G100*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J13" s="20">
@@ -10924,19 +11244,19 @@
         </is>
       </c>
       <c r="D14" s="27">
-        <f>ROUND(Inputs!B91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B101*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E14" s="27">
-        <f>ROUND(Inputs!C91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C101*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F14" s="27">
-        <f>ROUND(Inputs!D91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D101*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G14" s="27">
-        <f>ROUND(Inputs!E91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E101*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H14" s="24">
@@ -10944,7 +11264,7 @@
         <v/>
       </c>
       <c r="I14" s="24">
-        <f>ROUND(Inputs!G91*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G101*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J14" s="20">
@@ -10977,19 +11297,19 @@
         </is>
       </c>
       <c r="D15" s="27">
-        <f>ROUND(Inputs!B92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B102*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E15" s="27">
-        <f>ROUND(Inputs!C92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C102*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F15" s="27">
-        <f>ROUND(Inputs!D92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D102*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G15" s="27">
-        <f>ROUND(Inputs!E92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E102*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H15" s="24">
@@ -10997,7 +11317,7 @@
         <v/>
       </c>
       <c r="I15" s="24">
-        <f>ROUND(Inputs!G92*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G102*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J15" s="20">
@@ -11030,19 +11350,19 @@
         </is>
       </c>
       <c r="D16" s="27">
-        <f>ROUND(Inputs!B93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!B103*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="E16" s="27">
-        <f>ROUND(Inputs!C93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!C103*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="F16" s="27">
-        <f>ROUND(Inputs!D93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!D103*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="G16" s="27">
-        <f>ROUND(Inputs!E93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!E103*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="H16" s="24">
@@ -11050,7 +11370,7 @@
         <v/>
       </c>
       <c r="I16" s="24">
-        <f>ROUND(Inputs!G93*Local_Factor*FX*(1+Infra_Margin),-3)</f>
+        <f>ROUND(Inputs!G103*Local_Factor*FX*(1+Infra_Margin),-3)</f>
         <v/>
       </c>
       <c r="J16" s="20">
@@ -12113,7 +12433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -12367,16 +12687,16 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Connector go-live with a partner</t>
+          <t>Additional line of business after go-live</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>per connector</t>
+          <t>per line</t>
         </is>
       </c>
       <c r="C12" s="34">
-        <f>ROUND(Conn_Golive_Days*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(Days_per_LOB*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D12" s="20">
@@ -12384,28 +12704,28 @@
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>Conn_Golive_Days</f>
+        <f>Days_per_LOB</f>
         <v/>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>To confirm by management. A delivered connector (SMS gateway, CTPL provider, one insurer, one bank file layout, BIR EIS) taken live; the partner certifies its own side.</t>
+          <t>Product set-up, rating and tax lines, templates, testing.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Activation of the AML/CFT toolkit</t>
+          <t>New report or document template</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>one-time</t>
+          <t>per item (typical)</t>
         </is>
       </c>
       <c r="C13" s="34">
-        <f>ROUND(AML_Act_Days*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(Report_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D13" s="20">
@@ -12413,144 +12733,98 @@
         <v/>
       </c>
       <c r="E13" s="25">
-        <f>AML_Act_Days</f>
+        <f>Report_Days</f>
         <v/>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>To confirm by management. The toolkit is included in the software; this is the set-up effort. The compliance officer confirms the settings and loads the lists.</t>
+          <t>Small CR band; firm price after the impact note.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Activation of the IC compliance registers</t>
+          <t>On-site day (Metro Manila)</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>one-time</t>
+          <t>per consultant day</t>
         </is>
       </c>
       <c r="C14" s="34">
-        <f>ROUND(IC_Act_Days*Blended/Round_To,0)*Round_To</f>
+        <f>Rate_Onsite</f>
         <v/>
       </c>
       <c r="D14" s="20">
         <f>C14/FX</f>
         <v/>
       </c>
-      <c r="E14" s="25">
-        <f>IC_Act_Days</f>
-        <v/>
-      </c>
+      <c r="E14" s="25" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>To confirm by management. Registers included in the software; this is the set-up effort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Activation of the BIR pack</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>one-time</t>
-        </is>
-      </c>
-      <c r="C15" s="34">
-        <f>ROUND(BIR_Act_Days*Blended/Round_To,0)*Round_To</f>
-        <v/>
-      </c>
-      <c r="D15" s="20">
-        <f>C15/FX</f>
-        <v/>
-      </c>
-      <c r="E15" s="25">
-        <f>BIR_Act_Days</f>
-        <v/>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>To confirm by management. BIR forms, EOPT invoices, EIS and CAS pack included in the software; the tax adviser confirms the treatment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Dealer programme set-up</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>per programme</t>
-        </is>
-      </c>
-      <c r="C16" s="34">
-        <f>ROUND(Dealer_Prog_Days*Blended/Round_To,0)*Round_To</f>
-        <v/>
-      </c>
-      <c r="D16" s="20">
-        <f>C16/FX</f>
-        <v/>
-      </c>
-      <c r="E16" s="25">
-        <f>Dealer_Prog_Days</f>
-        <v/>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>To confirm by management. Dealer programmes are included in the software; this is the set-up of one programme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>Client brand pack</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>per pack</t>
-        </is>
-      </c>
-      <c r="C17" s="34">
-        <f>ROUND(Brand_Pack_Days*Blended/Round_To,0)*Round_To</f>
-        <v/>
-      </c>
-      <c r="D17" s="20">
-        <f>C17/FX</f>
-        <v/>
-      </c>
-      <c r="E17" s="25">
-        <f>Brand_Pack_Days</f>
-        <v/>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>To confirm by management. Branding is included in the software; a pack carrying third-party marks needs the owner's written permission.</t>
+          <t>Outside Metro Manila: travel, lodging and meals at cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Optional modules and partner services (confirmed by management on 04 October 2026): man-days x blended rate, rounded to PHP 10,000; the regulator's or partner's own fees are not included</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Price (PHP)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Price (USD)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Man-days</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Scope</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Additional line of business after go-live</t>
+          <t>Connector go-live with a partner</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>per line</t>
+          <t>per connector</t>
         </is>
       </c>
       <c r="C18" s="34">
-        <f>ROUND(Days_per_LOB*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(Conn_Golive_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D18" s="20">
@@ -12558,28 +12832,28 @@
         <v/>
       </c>
       <c r="E18" s="25">
-        <f>Days_per_LOB</f>
+        <f>Conn_Golive_Days</f>
         <v/>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Product set-up, rating and tax lines, templates, testing.</t>
+          <t>A delivered connector (SMS gateway, CTPL provider, one insurer, one bank file layout, BIR EIS) taken live: configuration, credential check, live test, support of the partner acceptance; the partner certifies its own side.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>New report or document template</t>
+          <t>Activation of the AML/CFT toolkit</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>per item (typical)</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C19" s="34">
-        <f>ROUND(Report_Days*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND(AML_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D19" s="20">
@@ -12587,179 +12861,571 @@
         <v/>
       </c>
       <c r="E19" s="25">
-        <f>Report_Days</f>
+        <f>AML_Act_Days</f>
         <v/>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Small CR band; firm price after the impact note.</t>
+          <t>The toolkit is included in the software; this is the set-up effort: risk factors and rules workshop, settings, first list loads, provider set-up, AMLC test file. The compliance officer confirms the settings and loads the lists.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>On-site day (Metro Manila)</t>
+          <t>Activation of the IC compliance registers</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>per consultant day</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C20" s="34">
-        <f>Rate_Onsite</f>
+        <f>ROUND(IC_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D20" s="20">
         <f>C20/FX</f>
         <v/>
       </c>
-      <c r="E20" s="25" t="inlineStr"/>
+      <c r="E20" s="25">
+        <f>IC_Act_Days</f>
+        <v/>
+      </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Outside Metro Manila: travel, lodging and meals at cost.</t>
+          <t>Registers included in the software; this is the set-up effort: licence and fit and proper register load, insurer certificates, complaints and breach settings, IC statement account mapping.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A28&amp;" tier"</f>
-        <v/>
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Activation of the BIR pack</t>
+        </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C21" s="34">
-        <f>Inputs!L28</f>
+        <f>ROUND(BIR_Act_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D21" s="20">
         <f>C21/FX</f>
         <v/>
       </c>
+      <c r="E21" s="25">
+        <f>BIR_Act_Days</f>
+        <v/>
+      </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Standard support is business hours (Monday to Friday, 08:00 to 18:00 Philippine time, excluding holidays). This adds round-the-clock response to Severity 1 incidents (production down or a core process stopped for all users).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A29&amp;" tier"</f>
-        <v/>
+          <t>BIR forms, EOPT invoices, EIS and CAS pack included in the software; this is the set-up effort: BIR and EOPT invoice settings, ATC mapping, DAT file dry run, CAS books pack. The tax adviser confirms the treatment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Dealer programme set-up</t>
+        </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>per programme</t>
         </is>
       </c>
       <c r="C22" s="34">
-        <f>Inputs!L29</f>
+        <f>ROUND(Dealer_Prog_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D22" s="20">
         <f>C22/FX</f>
         <v/>
       </c>
-      <c r="F22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A30&amp;" tier"</f>
-        <v/>
+      <c r="E22" s="25">
+        <f>Dealer_Prog_Days</f>
+        <v/>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Dealer programmes are included in the software; this is the set-up of one programme: channels, rates, subsidy, bank letter and the first upload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Client brand pack</t>
+        </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>per pack</t>
         </is>
       </c>
       <c r="C23" s="34">
-        <f>Inputs!L30</f>
+        <f>ROUND(Brand_Pack_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D23" s="20">
         <f>C23/FX</f>
         <v/>
       </c>
-      <c r="F23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="10">
-        <f>"24x7 Severity 1 support, "&amp;Inputs!A31&amp;" tier"</f>
-        <v/>
+      <c r="E23" s="25">
+        <f>Brand_Pack_Days</f>
+        <v/>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Branding is included in the software; this is one pack: theme, sign-in picture, document and e-mail branding, e-signature mapping, exported pack. A pack carrying third-party marks needs the owner's written permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>AMLC reporting file validation and portal test</t>
+        </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>per year, Year 1</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="C24" s="34">
-        <f>Inputs!L31</f>
+        <f>ROUND(AMLC_Val_Days*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="D24" s="20">
         <f>C24/FX</f>
         <v/>
       </c>
-      <c r="F24" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="E24" s="25">
+        <f>AMLC_Val_Days</f>
+        <v/>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>CTR and STR layout, institution and transaction codes confirmed with the AMLC, test file accepted in the AMLC portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>IC annual statement form alignment</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C25" s="34">
+        <f>ROUND(IC_Form_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>C25/FX</f>
+        <v/>
+      </c>
+      <c r="E25" s="25">
+        <f>IC_Form_Days</f>
+        <v/>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>The accountant working paper mapped to the IC form set in force for the year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>EOPT invoicing review with the broker tax adviser</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C26" s="34">
+        <f>ROUND(EOPT_Rev_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D26" s="20">
+        <f>C26/FX</f>
+        <v/>
+      </c>
+      <c r="E26" s="25">
+        <f>EOPT_Rev_Days</f>
+        <v/>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Registered invoice documents, supplementary wording, VAT treatment of each commission stream, ATP or CAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>BIR CAS registration support</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C27" s="34">
+        <f>ROUND(CAS_Reg_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D27" s="20">
+        <f>C27/FX</f>
+        <v/>
+      </c>
+      <c r="E27" s="25">
+        <f>CAS_Reg_Days</f>
+        <v/>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Books, system description and the Permit to Use filing prepared with the broker; the broker files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>BIR EIS enrolment and certification</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C28" s="34">
+        <f>ROUND(EIS_Enrol_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D28" s="20">
+        <f>C28/FX</f>
+        <v/>
+      </c>
+      <c r="E28" s="25">
+        <f>EIS_Enrol_Days</f>
+        <v/>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>EIS enrolment, signing certificate, final field list, production endpoint and certification of the connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>CTPL authentication and LTO interface certification</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C29" s="34">
+        <f>ROUND(CTPL_Cert_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D29" s="20">
+        <f>C29/FX</f>
+        <v/>
+      </c>
+      <c r="E29" s="25">
+        <f>CTPL_Cert_Days</f>
+        <v/>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Acceptance of the live requests by the accredited provider, COC series, LTO interface where the provider does not transmit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Insurer API onboarding, per insurer</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>per insurer</t>
+        </is>
+      </c>
+      <c r="C30" s="34">
+        <f>ROUND(Insurer_Onb_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>C30/FX</f>
+        <v/>
+      </c>
+      <c r="E30" s="25">
+        <f>Insurer_Onb_Days</f>
+        <v/>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint, credentials, field mapping and live test with one insurer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Bank payment file certification, per bank</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>per bank</t>
+        </is>
+      </c>
+      <c r="C31" s="34">
+        <f>ROUND(Bank_Cert_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D31" s="20">
+        <f>C31/FX</f>
+        <v/>
+      </c>
+      <c r="E31" s="25">
+        <f>Bank_Cert_Days</f>
+        <v/>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Layout validated against the bank specification and a test file accepted by the bank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>SMS or Viber gateway activation</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C32" s="34">
+        <f>ROUND(SMS_Act_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D32" s="20">
+        <f>C32/FX</f>
+        <v/>
+      </c>
+      <c r="E32" s="25">
+        <f>SMS_Act_Days</f>
+        <v/>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Sender name or short code, live credentials, templates and consent check tested with the gateway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Screening list provider onboarding</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>one-time</t>
+        </is>
+      </c>
+      <c r="C33" s="34">
+        <f>ROUND(Screen_Prov_Days*Blended/Round_To,0)*Round_To</f>
+        <v/>
+      </c>
+      <c r="D33" s="20">
+        <f>C33/FX</f>
+        <v/>
+      </c>
+      <c r="E33" s="25">
+        <f>Screen_Prov_Days</f>
+        <v/>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Provider contract data, API key, adapter test and first screening run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>24x7 Severity 1 support</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A28&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C36" s="34">
+        <f>Inputs!L28</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>C36/FX</f>
+        <v/>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Standard support is business hours (Monday to Friday, 08:00 to 18:00 Philippine time, excluding holidays). This adds round-the-clock response to Severity 1 incidents (production down or a core process stopped for all users).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A29&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C37" s="34">
+        <f>Inputs!L29</f>
+        <v/>
+      </c>
+      <c r="D37" s="20">
+        <f>C37/FX</f>
+        <v/>
+      </c>
+      <c r="F37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A30&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C38" s="34">
+        <f>Inputs!L30</f>
+        <v/>
+      </c>
+      <c r="D38" s="20">
+        <f>C38/FX</f>
+        <v/>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="10">
+        <f>"24x7 Severity 1 support, "&amp;Inputs!A31&amp;" tier"</f>
+        <v/>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>per year, Year 1</t>
+        </is>
+      </c>
+      <c r="C39" s="34">
+        <f>Inputs!L31</f>
+        <v/>
+      </c>
+      <c r="D39" s="20">
+        <f>C39/FX</f>
+        <v/>
+      </c>
+      <c r="F39" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Included in the standard implementation (no extra charge)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="26" t="inlineStr">
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
         <is>
           <t>Configuration of the company, branches, users and roles, insurers, commission rates, chart of accounts, banks and the included lines of business.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="26" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>Data load using the standard upload templates (about 50 templates in docs/package/05_Delivery/Upload_Templates), with the broker supplying clean data.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="26" t="inlineStr">
         <is>
           <t>Training days included for the tier (train-the-trainer), UAT support, go-live support and 4 weeks of hypercare.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="26" t="inlineStr">
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>Set-up of the environment set of the tier (Dev, UAT and Production; SIT as well for Large and Enterprise) and of Pre-Prod for the go-live rehearsal; hosting is billed separately. Deployment guidance when the broker hosts.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="26" t="inlineStr">
-        <is>
-          <t>Every module is included in the software price, including the AML/CFT toolkit, the IC compliance registers, the BIR pack, the integration framework with its connectors, dealer programmes and branding. Their activation and each connector go-live are the optional lines above (to confirm by management).</t>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>Every module is included in the software price, including the AML/CFT toolkit, the IC compliance registers, the BIR pack, the integration framework with its connectors, dealer programmes and branding. Their activation, each connector go-live and the regulator and partner services are the optional modules and partner services above, confirmed by management on 04 October 2026 as add-on items; no package total changes.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <printOptions gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12810,7 +13476,7 @@
     </row>
     <row r="4">
       <c r="A4" s="6">
-        <f>"Example 1: "&amp;Inputs!$B$99&amp;", "&amp;Inputs!$B$100&amp;" users, "&amp;Inputs!$B$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$B$102</f>
+        <f>"Example 1: "&amp;Inputs!$B$109&amp;", "&amp;Inputs!$B$110&amp;" users, "&amp;Inputs!$B$111&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$B$112</f>
         <v/>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -12877,7 +13543,7 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$B$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$B$111-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C7" s="20" t="n">
@@ -12908,7 +13574,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>MAX(0,MIN(Inputs!$B$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$B$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$B$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$B$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$B$110,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$B$110,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$B$110,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$B$110,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C8" s="20" t="n">
@@ -13042,27 +13708,27 @@
     </row>
     <row r="13">
       <c r="A13" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F13" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$B$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G13" s="34">
@@ -13118,27 +13784,27 @@
     </row>
     <row r="16">
       <c r="A16" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$B$102</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$B$112</f>
         <v/>
       </c>
       <c r="B16" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$B$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F16" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$B$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G16" s="34">
@@ -13157,23 +13823,23 @@
         </is>
       </c>
       <c r="B17" s="20">
-        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$B$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$B$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$B$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E17" s="20">
-        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$B$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F17" s="20">
-        <f>IF(Inputs!$B$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$B$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$B$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G17" s="34">
@@ -13192,7 +13858,7 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <f>Inputs!$B$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$B$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$B$106</f>
+        <f>Inputs!$B$114*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$B$115+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$B$116</f>
         <v/>
       </c>
       <c r="C18" s="20" t="n">
@@ -13434,7 +14100,7 @@
     </row>
     <row r="27">
       <c r="A27" s="6">
-        <f>"Example 2: "&amp;Inputs!$C$99&amp;", "&amp;Inputs!$C$100&amp;" users, "&amp;Inputs!$C$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$C$102</f>
+        <f>"Example 2: "&amp;Inputs!$C$109&amp;", "&amp;Inputs!$C$110&amp;" users, "&amp;Inputs!$C$111&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$C$112</f>
         <v/>
       </c>
       <c r="B27" s="7" t="n"/>
@@ -13501,7 +14167,7 @@
         </is>
       </c>
       <c r="B30" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$C$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$C$111-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C30" s="20" t="n">
@@ -13532,7 +14198,7 @@
         </is>
       </c>
       <c r="B31" s="20">
-        <f>MAX(0,MIN(Inputs!$C$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$C$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$C$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$C$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$C$110,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$C$110,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$C$110,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$C$110,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C31" s="20" t="n">
@@ -13666,27 +14332,27 @@
     </row>
     <row r="36">
       <c r="A36" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F36" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$C$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G36" s="34">
@@ -13742,27 +14408,27 @@
     </row>
     <row r="39">
       <c r="A39" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$C$102</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$C$112</f>
         <v/>
       </c>
       <c r="B39" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$C$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F39" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$C$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G39" s="34">
@@ -13781,23 +14447,23 @@
         </is>
       </c>
       <c r="B40" s="20">
-        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$C$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C40" s="20">
-        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$C$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D40" s="20">
-        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$C$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E40" s="20">
-        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$C$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F40" s="20">
-        <f>IF(Inputs!$C$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$C$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$C$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G40" s="34">
@@ -13816,7 +14482,7 @@
         </is>
       </c>
       <c r="B41" s="20">
-        <f>Inputs!$C$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$C$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$C$106</f>
+        <f>Inputs!$C$114*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$C$115+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$C$116</f>
         <v/>
       </c>
       <c r="C41" s="20" t="n">
@@ -14058,7 +14724,7 @@
     </row>
     <row r="50">
       <c r="A50" s="6">
-        <f>"Example 3: "&amp;Inputs!$D$99&amp;", "&amp;Inputs!$D$100&amp;" users, "&amp;Inputs!$D$101&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$D$102</f>
+        <f>"Example 3: "&amp;Inputs!$D$109&amp;", "&amp;Inputs!$D$110&amp;" users, "&amp;Inputs!$D$111&amp;" lines of business, tier "&amp;INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))&amp;", hosting: "&amp;Inputs!$D$112</f>
         <v/>
       </c>
       <c r="B50" s="7" t="n"/>
@@ -14125,7 +14791,7 @@
         </is>
       </c>
       <c r="B53" s="20">
-        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$D$101-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
+        <f>ROUND((INDEX(Inputs!$G$28:$G$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))+MAX(0,Inputs!$D$111-INDEX(Inputs!$H$28:$H$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1)))*Days_per_LOB)*Blended/Round_To,0)*Round_To</f>
         <v/>
       </c>
       <c r="C53" s="20" t="n">
@@ -14156,7 +14822,7 @@
         </is>
       </c>
       <c r="B54" s="20">
-        <f>MAX(0,MIN(Inputs!$D$100,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$D$100,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$D$100,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$D$100,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
+        <f>MAX(0,MIN(Inputs!$D$110,Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$D$28+MAX(0,MIN(Inputs!$D$110,Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$D$29+MAX(0,MIN(Inputs!$D$110,Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$D$30+MAX(0,MIN(Inputs!$D$110,Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$D$31</f>
         <v/>
       </c>
       <c r="C54" s="20" t="n">
@@ -14290,27 +14956,27 @@
     </row>
     <row r="59">
       <c r="A59" s="10">
-        <f>"Subscription ("&amp;MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
+        <f>"Subscription ("&amp;MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1)))&amp;" billable users)"</f>
         <v/>
       </c>
       <c r="B59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F59" s="20">
-        <f>(MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$100,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
+        <f>(MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$28)-Inputs!$B$28+1)*Inputs!$E$28+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$29)-Inputs!$B$29+1)*Inputs!$E$29+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$30)-Inputs!$B$30+1)*Inputs!$E$30+MAX(0,MIN(MAX(Inputs!$D$110,INDEX(Inputs!$F$28:$F$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))),Inputs!$C$31)-Inputs!$B$31+1)*Inputs!$E$31)*12*(1+Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G59" s="34">
@@ -14366,27 +15032,27 @@
     </row>
     <row r="62">
       <c r="A62" s="10">
-        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$D$102</f>
+        <f>"Hosting, environment set and Pre-Prod: "&amp;Inputs!$D$112</f>
         <v/>
       </c>
       <c r="B62" s="20">
-        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
+        <f>(SUMIFS(Infrastructure!$J$5:$J$20,Infrastructure!$A$5:$A$20,Inputs!$D$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(1-1)</f>
         <v/>
       </c>
       <c r="C62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(2-1)</f>
         <v/>
       </c>
       <c r="D62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(3-1)</f>
         <v/>
       </c>
       <c r="E62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(4-1)</f>
         <v/>
       </c>
       <c r="F62" s="20">
-        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$102,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
+        <f>(SUMIFS(Infrastructure!$K$5:$K$20,Infrastructure!$A$5:$A$20,Inputs!$D$112,Infrastructure!$B$5:$B$20,INDEX(Inputs!$A$28:$A$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))))*(1+Infra_Esc)^(5-1)</f>
         <v/>
       </c>
       <c r="G62" s="34">
@@ -14405,23 +15071,23 @@
         </is>
       </c>
       <c r="B63" s="20">
-        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
+        <f>IF(Inputs!$D$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(1-1),0)</f>
         <v/>
       </c>
       <c r="C63" s="20">
-        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
+        <f>IF(Inputs!$D$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(2-1),0)</f>
         <v/>
       </c>
       <c r="D63" s="20">
-        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
+        <f>IF(Inputs!$D$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(3-1),0)</f>
         <v/>
       </c>
       <c r="E63" s="20">
-        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
+        <f>IF(Inputs!$D$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(4-1),0)</f>
         <v/>
       </c>
       <c r="F63" s="20">
-        <f>IF(Inputs!$D$103="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$100,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
+        <f>IF(Inputs!$D$113="Yes",INDEX(Inputs!$L$28:$L$31,MATCH(Inputs!$D$110,Inputs!$B$28:$B$31,1))*(1+Esc)^(5-1),0)</f>
         <v/>
       </c>
       <c r="G63" s="34">
@@ -14440,7 +15106,7 @@
         </is>
       </c>
       <c r="B64" s="20">
-        <f>Inputs!$D$104*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$D$105+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$D$106</f>
+        <f>Inputs!$D$114*Rate_Trainer+ROUND(Mig_Days_Source*Blended/Round_To,0)*Round_To*Inputs!$D$115+ROUND(Int_Std_Days*Blended/Round_To,0)*Round_To*Inputs!$D$116</f>
         <v/>
       </c>
       <c r="C64" s="20" t="n">

</xml_diff>